<commit_message>
discussions on 0D and cooling data
</commit_message>
<xml_diff>
--- a/aysha/FittingTests v3.xlsx
+++ b/aysha/FittingTests v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\kkakosim\github\tamuq-chen-secarelab-receiver\aysha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAA99D8-5149-4706-8C07-ABF60BEAB030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC066E0-449C-4BEF-A319-5636E50E16A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0D" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <author>tc={1195A4A6-AC02-43B0-9B61-6F9ADFAE84CE}</author>
   </authors>
   <commentList>
-    <comment ref="B39" authorId="0" shapeId="0" xr:uid="{2C9673A5-534D-4FC2-A792-912F01D1091C}">
+    <comment ref="C39" authorId="0" shapeId="0" xr:uid="{2C9673A5-534D-4FC2-A792-912F01D1091C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -52,7 +52,7 @@
     10^A</t>
       </text>
     </comment>
-    <comment ref="D40" authorId="1" shapeId="0" xr:uid="{1195A4A6-AC02-43B0-9B61-6F9ADFAE84CE}">
+    <comment ref="E40" authorId="1" shapeId="0" xr:uid="{1195A4A6-AC02-43B0-9B61-6F9ADFAE84CE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="745">
   <si>
     <t>A</t>
   </si>
@@ -2352,6 +2352,21 @@
   </si>
   <si>
     <t>0D_v3 with NTU gas temperature</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>_v1</t>
+  </si>
+  <si>
+    <t>_v2</t>
+  </si>
+  <si>
+    <t>_v3</t>
+  </si>
+  <si>
+    <t>updated the objective function</t>
   </si>
 </sst>
 </file>
@@ -5839,10 +5854,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B39" dT="2025-07-23T05:22:20.02" personId="{276BCB23-7094-4A82-96C4-28630CE0F82D}" id="{2C9673A5-534D-4FC2-A792-912F01D1091C}">
+  <threadedComment ref="C39" dT="2025-07-23T05:22:20.02" personId="{276BCB23-7094-4A82-96C4-28630CE0F82D}" id="{2C9673A5-534D-4FC2-A792-912F01D1091C}">
     <text>10^A</text>
   </threadedComment>
-  <threadedComment ref="D40" dT="2025-07-23T05:38:31.92" personId="{276BCB23-7094-4A82-96C4-28630CE0F82D}" id="{1195A4A6-AC02-43B0-9B61-6F9ADFAE84CE}">
+  <threadedComment ref="E40" dT="2025-07-23T05:38:31.92" personId="{276BCB23-7094-4A82-96C4-28630CE0F82D}" id="{1195A4A6-AC02-43B0-9B61-6F9ADFAE84CE}">
     <text>10^</text>
   </threadedComment>
 </ThreadedComments>
@@ -5850,1335 +5865,1340 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:R108"/>
+  <dimension ref="A2:S110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="15" max="15" width="11.42578125" style="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="37.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="23"/>
+    <col min="16" max="16" width="11.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="37.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B2" s="23" t="s">
+        <v>740</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>670</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="O2" s="24" t="s">
+      <c r="P2" s="24" t="s">
         <v>729</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>717</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>718</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="C3" s="3">
         <v>1.24017003587548E-3</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>1.3974854403316901</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>1.6350743193202899</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>0.64</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1.1000000000000001</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1.2</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>0.8</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>19</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>23</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>27</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>1</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>0.4</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>499.47699999999998</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
+      <c r="C4" s="3">
         <v>9.7997522561352798E-4</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>1.4059359592048799</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2.4349761382305499</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>0.66</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>528.26599999999996</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
+      <c r="C5" s="3">
         <v>1.00002800832326E-4</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>1.3282580903963901</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>16.077659504854701</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>0.64</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>1</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>473.34</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
+      <c r="C6" s="3">
         <v>3.0774692673678297E-5</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>1.4802745324312101</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>19.9517218966303</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
+      <c r="C7" s="3">
         <v>3.1142977666936498E-3</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>1.2623131975854101</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>2.7362624606074699E-3</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>1</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>604.08600000000001</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
-      <c r="B8" s="3">
+      <c r="C8" s="3">
         <v>2.7615114875290401E-3</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>1.2412550503592701</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>1E-4</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>0.7</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
-      <c r="B9" s="3">
+      <c r="C9" s="3">
         <v>3.10648772630206E-3</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>1.2756696149129301</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>1E-4</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>0.63</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
-      <c r="B10" s="3">
+      <c r="C10" s="3">
         <v>8.6454867421348301E-5</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>1.64491004515391</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>12.0217117639568</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>1.2</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>500</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="3">
+      <c r="C11" s="3">
         <v>3.7125021077593002E-4</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>1.3930651456031</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>8.3576305806791193</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>0.64</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>480</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="R11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
-      <c r="B12" s="2">
+      <c r="C12" s="2">
         <v>2.6620817681730501E-5</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>1.4175004404023599</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>19.9997174906579</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>20</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>672</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="R12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>24</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>11</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>28</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>25612</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="R14" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>12</v>
       </c>
-      <c r="B15" s="2">
+      <c r="C15" s="2">
         <v>3.3035945380220997E-5</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>1.43770025274668</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>20</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>23</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>27</v>
       </c>
-      <c r="P15">
+      <c r="Q15">
         <v>469</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="R15" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13</v>
       </c>
-      <c r="P16" t="s">
+      <c r="Q16" t="s">
         <v>53</v>
       </c>
-      <c r="Q16" t="s">
+      <c r="R16" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>14</v>
       </c>
-      <c r="B17" s="2">
+      <c r="C17" s="2">
         <v>1.03191509408719E-5</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <v>1.4319313285872399</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>25.984272299692599</v>
       </c>
-      <c r="P17">
+      <c r="Q17">
         <v>465</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="R17" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>15</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="R18" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>16</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>0.84</v>
       </c>
-      <c r="P19">
+      <c r="Q19">
         <v>850</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="R19" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>17</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="R20" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>18</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>0.74</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>1.1000000000000001</v>
       </c>
-      <c r="P21">
+      <c r="Q21">
         <v>573</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="R21" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>19</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>0.64</v>
       </c>
-      <c r="P22">
+      <c r="Q22">
         <v>607</v>
       </c>
-      <c r="Q22" t="s">
+      <c r="R22" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>20</v>
       </c>
-      <c r="B23">
+      <c r="C23">
         <v>5.6058995390906102E-4</v>
       </c>
-      <c r="C23">
+      <c r="D23">
         <v>1.6106589591624401</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>9.910468968988089E-4</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>0.7</v>
       </c>
-      <c r="P23">
+      <c r="Q23">
         <v>502</v>
       </c>
-      <c r="Q23" t="s">
+      <c r="R23" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>21</v>
       </c>
-      <c r="B24" s="2">
+      <c r="C24" s="2">
         <v>1.0024299213338499E-5</v>
       </c>
-      <c r="C24">
+      <c r="D24">
         <v>2.9323882617891202</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>1E-4</v>
       </c>
-      <c r="L24">
+      <c r="M24">
         <v>4.4000000000000004</v>
       </c>
-      <c r="P24">
+      <c r="Q24">
         <v>1641</v>
       </c>
-      <c r="Q24" t="s">
+      <c r="R24" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>22</v>
       </c>
-      <c r="B25" s="2">
+      <c r="C25" s="2">
         <v>2.0887059774144901E-5</v>
       </c>
-      <c r="C25">
+      <c r="D25">
         <v>2.5052539496126101</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>1.8829968719792201E-2</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>1</v>
       </c>
-      <c r="P25">
+      <c r="Q25">
         <v>1071</v>
       </c>
-      <c r="Q25" t="s">
+      <c r="R25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>1</v>
       </c>
-      <c r="P26">
+      <c r="Q26">
         <v>1892</v>
       </c>
-      <c r="Q26" t="s">
+      <c r="R26" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
-      <c r="B27">
+      <c r="C27">
         <v>2.1591196456141501E-4</v>
       </c>
-      <c r="C27">
+      <c r="D27">
         <v>1.7189995203791599</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>1.20209817420813</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>0.9</v>
       </c>
-      <c r="P27">
+      <c r="Q27">
         <v>1354</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
-      <c r="B28">
+      <c r="C28">
         <v>3.0880065502844102E-4</v>
       </c>
-      <c r="C28">
+      <c r="D28">
         <v>1.7074022707650001</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>3.7186641941726502E-4</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>0.85</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>26</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>0.7</v>
       </c>
-      <c r="P29">
+      <c r="Q29">
         <v>502</v>
       </c>
-      <c r="Q29" t="s">
+      <c r="R29" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>27</v>
       </c>
-      <c r="B30">
+      <c r="C30">
         <v>4.60311808037377E-4</v>
       </c>
-      <c r="C30">
+      <c r="D30">
         <v>1.66187478217667</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>1.3738648256894E-4</v>
       </c>
-      <c r="P30">
+      <c r="Q30">
         <v>502</v>
       </c>
-      <c r="Q30" t="s">
+      <c r="R30" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>28</v>
       </c>
-      <c r="B31">
+      <c r="C31">
         <v>5.86247778425387E-4</v>
       </c>
-      <c r="C31">
+      <c r="D31">
         <v>1.6630696101604501</v>
       </c>
-      <c r="D31" s="2">
+      <c r="E31" s="2">
         <v>9.39537377217747E-5</v>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>0.6</v>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <v>522</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>29</v>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <v>522</v>
       </c>
-      <c r="Q32" t="s">
+      <c r="R32" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30</v>
       </c>
-      <c r="B33">
+      <c r="C33">
         <v>2.8727643386340098E-4</v>
       </c>
-      <c r="C33">
+      <c r="D33">
         <v>1.5904189645704501</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>1.0263197679569199E-4</v>
       </c>
-      <c r="N33">
+      <c r="O33">
         <v>0</v>
       </c>
-      <c r="P33">
+      <c r="Q33">
         <v>563</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>31</v>
       </c>
-      <c r="B34">
+      <c r="C34">
         <v>3.0928717643758302E-4</v>
       </c>
-      <c r="C34">
+      <c r="D34">
         <v>1.5965904733758101</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>2.4080124471630401E-4</v>
       </c>
-      <c r="F34">
+      <c r="G34">
         <v>1</v>
       </c>
-      <c r="G34">
+      <c r="H34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="P34">
+      <c r="Q34">
         <v>461</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>32</v>
       </c>
-      <c r="B35">
+      <c r="C35">
         <v>2.4681495887314401E-4</v>
       </c>
-      <c r="C35">
+      <c r="D35">
         <v>1.6624759537039799</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>1.7341179006468701E-4</v>
       </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
         <v>72</v>
       </c>
-      <c r="P35">
+      <c r="Q35">
         <v>482</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>33</v>
       </c>
-      <c r="E36">
+      <c r="F36">
         <v>0.64</v>
       </c>
-      <c r="K36" t="s">
+      <c r="L36" t="s">
         <v>27</v>
       </c>
-      <c r="P36">
+      <c r="Q36">
         <v>586</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>34</v>
       </c>
-      <c r="E37">
+      <c r="F37">
         <v>0.75</v>
       </c>
-      <c r="P37">
+      <c r="Q37">
         <v>550</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="N38">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O38">
         <v>0</v>
       </c>
-      <c r="Q38" s="20" t="s">
+      <c r="R38" s="20" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>35</v>
       </c>
-      <c r="B39">
+      <c r="C39">
         <v>-1.5880535011177801</v>
       </c>
-      <c r="C39">
+      <c r="D39">
         <v>0.65091494933399197</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>3.6666969736259901E-2</v>
       </c>
-      <c r="E39">
+      <c r="F39">
         <v>1</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>0.7</v>
       </c>
-      <c r="I39">
+      <c r="J39">
         <v>7.8E-2</v>
       </c>
-      <c r="P39">
+      <c r="Q39">
         <v>1140</v>
       </c>
-      <c r="Q39" t="s">
+      <c r="R39" t="s">
         <v>662</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>36</v>
       </c>
-      <c r="B40">
+      <c r="C40">
         <v>-1.62557011221157</v>
       </c>
-      <c r="C40">
+      <c r="D40">
         <v>0.64353970719628895</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>-5</v>
       </c>
-      <c r="L40">
+      <c r="M40">
         <v>3</v>
       </c>
-      <c r="P40">
+      <c r="Q40">
         <v>975</v>
       </c>
-      <c r="Q40" t="s">
+      <c r="R40" t="s">
         <v>666</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>37</v>
       </c>
-      <c r="L41">
+      <c r="M41">
         <v>1</v>
       </c>
-      <c r="P41">
+      <c r="Q41">
         <v>1140</v>
       </c>
-      <c r="Q41" t="s">
+      <c r="R41" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>38</v>
       </c>
-      <c r="B42">
+      <c r="C42">
         <v>-1.62633085814944</v>
       </c>
-      <c r="C42">
+      <c r="D42">
         <v>0.64384726379398405</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <v>-4.2152141852378398</v>
       </c>
-      <c r="E42">
+      <c r="F42">
         <v>1.2</v>
       </c>
-      <c r="M42">
+      <c r="N42">
         <v>3</v>
       </c>
-      <c r="P42">
+      <c r="Q42">
         <v>975</v>
       </c>
-      <c r="Q42" t="s">
+      <c r="R42" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>39</v>
       </c>
-      <c r="B43">
+      <c r="C43">
         <v>-1.62557011221157</v>
       </c>
-      <c r="C43">
+      <c r="D43">
         <v>0.64353970719628895</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>-5</v>
       </c>
-      <c r="E43">
+      <c r="F43">
         <v>1</v>
       </c>
-      <c r="L43">
+      <c r="M43">
         <v>3</v>
       </c>
-      <c r="M43">
+      <c r="N43">
         <v>1</v>
       </c>
-      <c r="P43">
+      <c r="Q43">
         <v>975</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>40</v>
       </c>
-      <c r="B44">
+      <c r="C44">
         <v>-0.21738961927643199</v>
       </c>
-      <c r="C44">
+      <c r="D44">
         <v>0.224136849475497</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>-4.38627582837346</v>
       </c>
-      <c r="E44">
+      <c r="F44">
         <v>1</v>
       </c>
-      <c r="P44">
+      <c r="Q44">
         <v>1496</v>
       </c>
-      <c r="Q44" t="s">
+      <c r="R44" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>41</v>
       </c>
-      <c r="B45">
+      <c r="C45">
         <v>-0.120453173998853</v>
       </c>
-      <c r="C45">
+      <c r="D45">
         <v>8.2527627411642504E-2</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>-5</v>
       </c>
-      <c r="E45">
+      <c r="F45">
         <v>0.7</v>
       </c>
-      <c r="P45">
+      <c r="Q45">
         <v>1027</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>42</v>
       </c>
-      <c r="B46">
+      <c r="C46">
         <v>-6.3694404355623402E-2</v>
       </c>
-      <c r="C46">
+      <c r="D46">
         <v>6.9338798965457998E-2</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>-3.66322327238499</v>
       </c>
-      <c r="L46">
+      <c r="M46">
         <v>2</v>
       </c>
-      <c r="P46">
+      <c r="Q46">
         <v>999</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>43</v>
       </c>
-      <c r="B47">
+      <c r="C47">
         <v>-5.6187532274797197E-2</v>
       </c>
-      <c r="C47">
+      <c r="D47">
         <v>6.7192097637876202E-2</v>
       </c>
-      <c r="D47">
+      <c r="E47">
         <v>-3.85853069192695</v>
       </c>
-      <c r="P47">
+      <c r="Q47">
         <v>999</v>
       </c>
-      <c r="Q47" t="s">
+      <c r="R47" t="s">
         <v>674</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B48">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="C48">
         <v>-0.59913658322029595</v>
       </c>
-      <c r="C48">
+      <c r="D48">
         <v>0.23267951536977999</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>-4.54729113095385</v>
       </c>
-      <c r="P48">
+      <c r="Q48">
         <v>1050</v>
       </c>
-      <c r="Q48" t="s">
+      <c r="R48" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="49" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B49">
+    <row r="49" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C49">
         <v>-3.0218416280894E-2</v>
       </c>
-      <c r="C49">
+      <c r="D49">
         <v>5.6553370855678999E-2</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>-5</v>
       </c>
-      <c r="L49" t="s">
+      <c r="M49" t="s">
         <v>678</v>
       </c>
-      <c r="P49">
+      <c r="Q49">
         <v>996</v>
       </c>
     </row>
-    <row r="50" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B50">
+    <row r="50" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C50">
         <v>2.32366143478863</v>
       </c>
-      <c r="C50">
+      <c r="D50">
         <v>5.2381129172708499E-2</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>1.15176621671389</v>
       </c>
-      <c r="L50" t="s">
+      <c r="M50" t="s">
         <v>679</v>
       </c>
-      <c r="P50">
+      <c r="Q50">
         <v>1195</v>
       </c>
-      <c r="Q50" t="s">
+      <c r="R50" t="s">
         <v>680</v>
       </c>
     </row>
-    <row r="51" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B51">
+    <row r="51" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C51">
         <v>-0.11531413827813</v>
       </c>
-      <c r="C51">
+      <c r="D51">
         <v>0.110780162848843</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>-5</v>
       </c>
-      <c r="F51">
+      <c r="G51">
         <v>1.1499999999999999</v>
       </c>
-      <c r="L51" t="s">
+      <c r="M51" t="s">
         <v>681</v>
       </c>
-      <c r="P51">
+      <c r="Q51">
         <v>1049</v>
       </c>
     </row>
-    <row r="52" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B52">
+    <row r="52" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C52">
         <v>-5.9825795140801101E-2</v>
       </c>
-      <c r="C52">
+      <c r="D52">
         <v>8.3298389397967201E-2</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>-4.7822766948941098</v>
       </c>
-      <c r="F52">
+      <c r="G52">
         <v>1.1000000000000001</v>
       </c>
-      <c r="P52">
+      <c r="Q52">
         <v>1016</v>
       </c>
     </row>
-    <row r="53" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B53">
+    <row r="53" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C53">
         <v>0.163215104178386</v>
       </c>
-      <c r="C53">
+      <c r="D53">
         <v>0.110019492778361</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>-5</v>
       </c>
-      <c r="E53">
+      <c r="F53">
         <v>1</v>
       </c>
-      <c r="P53">
+      <c r="Q53">
         <v>1882</v>
       </c>
     </row>
-    <row r="54" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B54">
+    <row r="54" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C54">
         <v>0.16620523432742201</v>
       </c>
-      <c r="C54">
+      <c r="D54">
         <v>0.10949611407786</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>-1.95188474207697</v>
       </c>
-      <c r="P54">
+      <c r="Q54">
         <v>1880</v>
       </c>
-      <c r="Q54" t="s">
+      <c r="R54" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="55" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B55">
+    <row r="55" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C55">
         <v>0.113337590003834</v>
       </c>
-      <c r="C55">
+      <c r="D55">
         <v>0.113912815280584</v>
       </c>
-      <c r="D55">
+      <c r="E55">
         <v>-3.17711423761659</v>
       </c>
-      <c r="F55">
+      <c r="G55">
         <v>1</v>
       </c>
-      <c r="P55">
+      <c r="Q55">
         <v>1692</v>
       </c>
     </row>
-    <row r="56" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B56">
+    <row r="56" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C56">
         <v>0.115547627813837</v>
       </c>
-      <c r="C56">
+      <c r="D56">
         <v>0.113073002583607</v>
       </c>
-      <c r="D56">
+      <c r="E56">
         <v>-4.5277566109866303</v>
       </c>
-      <c r="P56">
+      <c r="Q56">
         <v>1692</v>
       </c>
-      <c r="Q56" t="s">
+      <c r="R56" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="57" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B57">
+    <row r="57" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C57">
         <v>-3.3149389346669902E-2</v>
       </c>
-      <c r="C57">
+      <c r="D57">
         <v>5.74856315526577E-2</v>
       </c>
-      <c r="D57">
+      <c r="E57">
         <v>-5</v>
       </c>
-      <c r="E57">
+      <c r="F57">
         <v>0.7</v>
       </c>
-      <c r="P57">
+      <c r="Q57">
         <v>996</v>
       </c>
     </row>
-    <row r="58" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="E58">
+    <row r="58" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="F58">
         <v>1</v>
       </c>
-      <c r="Q58" t="s">
+      <c r="R58" t="s">
         <v>684</v>
       </c>
     </row>
-    <row r="59" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B59">
+    <row r="59" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C59">
         <v>0.250054010925023</v>
       </c>
-      <c r="C59">
+      <c r="D59">
         <v>9.0017378931107103E-2</v>
       </c>
-      <c r="D59">
+      <c r="E59">
         <v>-3.5197283757326399</v>
       </c>
-      <c r="P59">
+      <c r="Q59">
         <v>1746</v>
       </c>
-      <c r="Q59" t="s">
+      <c r="R59" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="60" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B60">
+    <row r="60" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C60">
         <v>-1.44059076725918</v>
       </c>
-      <c r="C60">
+      <c r="D60">
         <v>0.67522154899549303</v>
       </c>
-      <c r="D60">
+      <c r="E60">
         <v>-4.8807740743608301</v>
       </c>
-      <c r="P60">
+      <c r="Q60">
         <v>1574</v>
       </c>
-      <c r="Q60" t="s">
+      <c r="R60" t="s">
         <v>688</v>
       </c>
     </row>
-    <row r="61" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B61">
+    <row r="61" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C61">
         <v>-1.21144890336943</v>
       </c>
-      <c r="C61">
+      <c r="D61">
         <v>0.594262978875436</v>
       </c>
-      <c r="D61">
+      <c r="E61">
         <v>-5</v>
       </c>
-      <c r="H61">
+      <c r="I61">
         <v>1</v>
       </c>
-      <c r="P61">
+      <c r="Q61">
         <v>2108</v>
       </c>
     </row>
-    <row r="62" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B62">
+    <row r="62" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C62">
         <v>-1.2070813277479999</v>
       </c>
-      <c r="C62">
+      <c r="D62">
         <v>0.49223109727618702</v>
       </c>
-      <c r="D62">
+      <c r="E62">
         <v>-5</v>
       </c>
-      <c r="E62">
+      <c r="F62">
         <v>0.7</v>
       </c>
-      <c r="H62">
+      <c r="I62">
         <v>0.7</v>
       </c>
-      <c r="P62">
+      <c r="Q62">
         <v>1309</v>
       </c>
     </row>
-    <row r="63" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B63">
+    <row r="63" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C63">
         <v>-1.0012021396300801</v>
       </c>
-      <c r="C63">
+      <c r="D63">
         <v>0.40143186621960603</v>
       </c>
-      <c r="D63">
+      <c r="E63">
         <v>-5</v>
       </c>
-      <c r="P63">
+      <c r="Q63">
         <v>994</v>
       </c>
     </row>
-    <row r="64" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B64">
+    <row r="64" spans="3:18" x14ac:dyDescent="0.25">
+      <c r="C64">
         <v>-4.4248727373665302</v>
       </c>
-      <c r="C64">
+      <c r="D64">
         <v>2.0054297178263898</v>
       </c>
-      <c r="D64">
+      <c r="E64">
         <v>-0.92802622567503801</v>
       </c>
-      <c r="P64">
+      <c r="Q64">
         <v>1528</v>
       </c>
-      <c r="Q64" t="s">
+      <c r="R64" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B65">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C65">
         <v>-1.0608132419307801</v>
       </c>
-      <c r="C65">
+      <c r="D65">
         <v>0.415984490245218</v>
       </c>
-      <c r="D65">
+      <c r="E65">
         <v>-4.9695269901766101</v>
       </c>
-      <c r="L65" t="s">
+      <c r="M65" t="s">
         <v>681</v>
       </c>
-      <c r="P65">
+      <c r="Q65">
         <v>1167</v>
       </c>
-      <c r="Q65" t="s">
+      <c r="R65" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B66">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C66">
         <v>-1.1261289140861099</v>
       </c>
-      <c r="C66">
+      <c r="D66">
         <v>0.47186731215250699</v>
       </c>
-      <c r="D66">
+      <c r="E66">
         <v>-4.5038498068435002</v>
       </c>
-      <c r="F66">
+      <c r="G66">
         <v>1.1499999999999999</v>
       </c>
-      <c r="P66">
+      <c r="Q66">
         <v>1002</v>
       </c>
-      <c r="Q66" t="s">
+      <c r="R66" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B67">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C67">
         <v>-1.2035253749880399</v>
       </c>
-      <c r="C67">
+      <c r="D67">
         <v>0.49275278422355101</v>
       </c>
-      <c r="D67">
+      <c r="E67">
         <v>-4.83529833670908</v>
       </c>
-      <c r="P67">
+      <c r="Q67">
         <v>1121</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B68">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C68">
         <v>-1.44395477402174</v>
       </c>
-      <c r="C68">
+      <c r="D68">
         <v>0.49278508137217503</v>
       </c>
-      <c r="D68">
+      <c r="E68">
         <v>-4.59924882828237</v>
       </c>
-      <c r="P68">
+      <c r="Q68">
         <v>1121</v>
       </c>
-      <c r="Q68" t="s">
+      <c r="R68" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="69" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="O69" s="25"/>
-    </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B70">
+    <row r="69" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="25"/>
+      <c r="P69" s="25"/>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B70" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="C70">
         <v>-1.2038</v>
       </c>
-      <c r="C70">
+      <c r="D70">
         <v>0.4929</v>
       </c>
-      <c r="D70">
+      <c r="E70">
         <v>-4.9325999999999999</v>
       </c>
-      <c r="L70" t="s">
+      <c r="M70" t="s">
         <v>727</v>
       </c>
-      <c r="Q70" t="s">
+      <c r="R70" t="s">
         <v>713</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B71">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C71">
         <v>-0.70223850678134803</v>
       </c>
-      <c r="C71">
+      <c r="D71">
         <v>0.25645673662077101</v>
       </c>
-      <c r="D71">
+      <c r="E71">
         <v>-4.9512972108205302</v>
       </c>
-      <c r="Q71" t="s">
+      <c r="R71" t="s">
         <v>714</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E72">
-        <v>1</v>
-      </c>
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F72">
         <v>1</v>
       </c>
@@ -7188,443 +7208,479 @@
       <c r="H72">
         <v>1</v>
       </c>
-      <c r="P72">
+      <c r="I72">
+        <v>1</v>
+      </c>
+      <c r="Q72">
         <v>1147</v>
       </c>
-      <c r="Q72" t="s">
+      <c r="R72" t="s">
         <v>715</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B73">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C73">
         <v>-1.8904675242014499</v>
       </c>
-      <c r="C73">
+      <c r="D73">
         <v>0.78604681017162004</v>
       </c>
-      <c r="D73">
+      <c r="E73">
         <v>-4.8087781051542704</v>
       </c>
-      <c r="F73">
+      <c r="G73">
         <v>1.1499999999999999</v>
       </c>
-      <c r="G73">
+      <c r="H73">
         <v>1</v>
       </c>
-      <c r="H73">
+      <c r="I73">
         <v>0.7</v>
       </c>
-      <c r="P73">
+      <c r="Q73">
         <v>1165</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>4</v>
       </c>
-      <c r="B74">
+      <c r="C74">
         <v>-1.8904675242014499</v>
       </c>
-      <c r="C74">
+      <c r="D74">
         <v>0.78604681017162004</v>
       </c>
-      <c r="D74">
+      <c r="E74">
         <v>-4.8087781051542704</v>
       </c>
-      <c r="G74">
+      <c r="H74">
         <v>1.1499999999999999</v>
       </c>
-      <c r="P74">
+      <c r="Q74">
         <v>1165</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>5</v>
       </c>
-      <c r="B75">
+      <c r="C75">
         <v>-2.92555847278929</v>
       </c>
-      <c r="C75">
+      <c r="D75">
         <v>1.1553271728060299</v>
       </c>
-      <c r="D75">
+      <c r="E75">
         <v>-5</v>
       </c>
-      <c r="P75">
+      <c r="Q75">
         <v>1110</v>
       </c>
-      <c r="Q75" t="s">
+      <c r="R75" t="s">
         <v>688</v>
       </c>
-      <c r="R75" t="s">
+      <c r="S75" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>6</v>
       </c>
-      <c r="B76" s="23">
+      <c r="C76" s="23">
         <v>-4.2861727192109598</v>
       </c>
-      <c r="C76">
+      <c r="D76">
         <v>1.98660254327817</v>
       </c>
-      <c r="D76">
+      <c r="E76">
         <v>-5</v>
       </c>
-      <c r="P76">
+      <c r="Q76">
         <v>1613</v>
       </c>
-      <c r="Q76" t="s">
+      <c r="R76" t="s">
         <v>716</v>
       </c>
-      <c r="R76" t="s">
+      <c r="S76" t="s">
         <v>720</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="22" t="s">
         <v>721</v>
       </c>
-      <c r="E77">
+      <c r="B77" s="22"/>
+      <c r="F77">
         <v>0.7</v>
       </c>
-      <c r="R77" t="s">
+      <c r="S77" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>7</v>
       </c>
-      <c r="E78">
+      <c r="F78">
         <v>0.8</v>
       </c>
-      <c r="F78">
+      <c r="G78">
         <v>1</v>
       </c>
-      <c r="P78">
+      <c r="Q78">
         <v>1101</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E79">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="F79">
         <v>0.75</v>
       </c>
-      <c r="P79">
+      <c r="Q79">
         <v>1152</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E80">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="F80">
         <v>0.72499999999999998</v>
       </c>
-      <c r="G80">
+      <c r="H80">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="H81">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="I81">
         <v>0.9</v>
       </c>
-      <c r="P81">
+      <c r="Q81">
         <v>1237</v>
       </c>
-      <c r="R81" t="s">
+      <c r="S81" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q82" t="s">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="R82" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="F83">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="G83">
         <v>0.9</v>
       </c>
-      <c r="P83">
+      <c r="Q83">
         <v>1311</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="H84">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="I84">
         <v>0.85</v>
       </c>
-      <c r="P84">
+      <c r="Q84">
         <v>1255</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E85">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="F85">
         <v>0.7</v>
       </c>
-      <c r="P85">
+      <c r="Q85">
         <v>1318</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="H86">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="I86">
         <v>0.8</v>
       </c>
-      <c r="P86">
+      <c r="Q86">
         <v>1337</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="H87">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="I87">
         <v>0.75</v>
       </c>
-      <c r="P87">
+      <c r="Q87">
         <v>1368</v>
       </c>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>18</v>
       </c>
-      <c r="F88">
+      <c r="G88">
         <v>0.85</v>
       </c>
-      <c r="G88">
+      <c r="H88">
         <v>1.05</v>
       </c>
-      <c r="P88">
+      <c r="Q88">
         <v>1463</v>
       </c>
-      <c r="R88" t="s">
+      <c r="S88" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>19</v>
       </c>
-      <c r="P89">
+      <c r="Q89">
         <v>2704</v>
       </c>
-      <c r="Q89" t="s">
+      <c r="R89" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>20</v>
       </c>
-      <c r="E90">
+      <c r="F90">
         <v>0.9</v>
       </c>
-      <c r="P90">
+      <c r="Q90">
         <v>1939</v>
       </c>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>21</v>
       </c>
-      <c r="F91">
+      <c r="G91">
         <v>1</v>
       </c>
-      <c r="G91">
+      <c r="H91">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H91">
+      <c r="I91">
         <v>0.8</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>22</v>
       </c>
-      <c r="E92">
+      <c r="F92">
         <v>0.95</v>
       </c>
-      <c r="P92">
+      <c r="Q92">
         <v>1439</v>
       </c>
-      <c r="R92" t="s">
+      <c r="S92" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>23</v>
       </c>
-      <c r="G93">
+      <c r="H93">
         <v>1.1499999999999999</v>
       </c>
-      <c r="P93">
+      <c r="Q93">
         <v>1399</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>24</v>
       </c>
-      <c r="E94">
+      <c r="F94">
         <v>1</v>
       </c>
-      <c r="P94">
+      <c r="Q94">
         <v>1256</v>
       </c>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>25</v>
       </c>
-      <c r="E95">
+      <c r="F95">
         <v>1.1000000000000001</v>
       </c>
-      <c r="P95">
+      <c r="Q95">
         <v>1052</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>26</v>
       </c>
-      <c r="E96">
+      <c r="F96">
         <v>1.05</v>
       </c>
-      <c r="P96">
+      <c r="Q96">
         <v>1139</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="L97" t="s">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M97" t="s">
         <v>728</v>
       </c>
-      <c r="P97">
+      <c r="Q97">
         <v>872</v>
       </c>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="O98" s="23" t="s">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="P98" s="23" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>29</v>
       </c>
-      <c r="O99" s="23" t="s">
+      <c r="P99" s="23" t="s">
         <v>731</v>
       </c>
-      <c r="P99">
+      <c r="Q99">
         <v>1216</v>
       </c>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>30</v>
       </c>
-      <c r="E100">
+      <c r="F100">
         <v>1</v>
       </c>
-      <c r="P100">
+      <c r="Q100">
         <v>896</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>31</v>
       </c>
-      <c r="H101">
+      <c r="I101">
         <v>0.7</v>
       </c>
-      <c r="P101">
+      <c r="Q101">
         <v>938</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>1</v>
       </c>
-      <c r="P102">
+      <c r="B102" s="23" t="s">
+        <v>741</v>
+      </c>
+      <c r="Q102">
         <v>2033</v>
       </c>
-      <c r="Q102" t="s">
+      <c r="R102" t="s">
         <v>732</v>
       </c>
-      <c r="R102" t="s">
+      <c r="S102" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>32</v>
       </c>
-      <c r="E103">
+      <c r="B103" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="F103">
         <v>0.8</v>
       </c>
-      <c r="Q103" t="s">
+      <c r="R103" t="s">
         <v>734</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2</v>
       </c>
-      <c r="P104">
+      <c r="B104" s="23" t="s">
+        <v>741</v>
+      </c>
+      <c r="Q104">
         <v>1322</v>
       </c>
-      <c r="Q104" s="23" t="s">
+      <c r="R104" s="23" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>33</v>
       </c>
-      <c r="E105">
+      <c r="B105" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="F105">
         <v>1</v>
       </c>
-      <c r="P105">
+      <c r="Q105">
         <v>938</v>
       </c>
-      <c r="Q105" s="23" t="s">
+      <c r="R105" s="23" t="s">
         <v>734</v>
       </c>
-      <c r="R105" s="25" t="s">
+      <c r="S105" s="25" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>34</v>
       </c>
-      <c r="P106">
+      <c r="B106" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="Q106">
         <v>938</v>
       </c>
-      <c r="Q106" t="s">
+      <c r="R106" t="s">
         <v>736</v>
       </c>
-      <c r="R106" t="s">
+      <c r="S106" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>35</v>
       </c>
-      <c r="P107">
+      <c r="B107" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="Q107">
         <v>925</v>
       </c>
-      <c r="Q107" t="s">
+      <c r="R107" t="s">
         <v>738</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2</v>
       </c>
-      <c r="P108">
+      <c r="B108" s="23" t="s">
+        <v>743</v>
+      </c>
+      <c r="Q108">
         <v>943</v>
       </c>
-      <c r="Q108" t="s">
+      <c r="R108" t="s">
         <v>739</v>
+      </c>
+    </row>
+    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>4</v>
+      </c>
+      <c r="Q110">
+        <v>0.06</v>
+      </c>
+      <c r="R110" s="23" t="s">
+        <v>744</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated v3 to run with v4 corrections
</commit_message>
<xml_diff>
--- a/aysha/FittingTests v3.xlsx
+++ b/aysha/FittingTests v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\kkakosim\github\tamuq-chen-secarelab-receiver\aysha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC066E0-449C-4BEF-A319-5636E50E16A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F8773D-E160-4CBE-9BF5-BC99F7C3FA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="746">
   <si>
     <t>A</t>
   </si>
@@ -2367,6 +2367,9 @@
   </si>
   <si>
     <t>updated the objective function</t>
+  </si>
+  <si>
+    <t>Tfilm for Tgas and weighted Taveraged for the solid</t>
   </si>
 </sst>
 </file>
@@ -5865,7 +5868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:S110"/>
+  <dimension ref="A2:S111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="23"/>
@@ -7681,6 +7684,17 @@
       </c>
       <c r="R110" s="23" t="s">
         <v>744</v>
+      </c>
+    </row>
+    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>5</v>
+      </c>
+      <c r="Q111">
+        <v>0.05</v>
+      </c>
+      <c r="R111" t="s">
+        <v>745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates to _v3 and v4
_v3 same plots with v4 including the cooling results
_v4 use the same Io from import
</commit_message>
<xml_diff>
--- a/aysha/FittingTests v3.xlsx
+++ b/aysha/FittingTests v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\kkakosim\github\tamuq-chen-secarelab-receiver\aysha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F8773D-E160-4CBE-9BF5-BC99F7C3FA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B23D3CE-AE50-4D97-AFC6-605C5039AEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="750">
   <si>
     <t>A</t>
   </si>
@@ -2354,9 +2354,6 @@
     <t>0D_v3 with NTU gas temperature</t>
   </si>
   <si>
-    <t>mode</t>
-  </si>
-  <si>
     <t>_v1</t>
   </si>
   <si>
@@ -2366,10 +2363,25 @@
     <t>_v3</t>
   </si>
   <si>
+    <t>_v4</t>
+  </si>
+  <si>
     <t>updated the objective function</t>
   </si>
   <si>
     <t>Tfilm for Tgas and weighted Taveraged for the solid</t>
+  </si>
+  <si>
+    <t>include cooling, and focusing on the 0D parameters</t>
+  </si>
+  <si>
+    <t>solid profile not bad, but gas and time not good</t>
+  </si>
+  <si>
+    <t>similar plotting style with v4, included cooling output</t>
+  </si>
+  <si>
+    <t>model</t>
   </si>
 </sst>
 </file>
@@ -5868,18 +5880,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:S111"/>
+  <dimension ref="A2:S114"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.140625" style="23"/>
+    <col min="1" max="1" width="9.140625" style="23"/>
     <col min="16" max="16" width="11.42578125" style="23" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="46.85546875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="37.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="23" t="s">
-        <v>740</v>
+      <c r="A2" s="23" t="s">
+        <v>749</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>0</v>
@@ -5934,7 +5946,7 @@
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="3">
@@ -5981,7 +5993,7 @@
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" s="3">
@@ -6004,7 +6016,7 @@
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" s="3">
@@ -6030,7 +6042,7 @@
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="B6">
         <v>4</v>
       </c>
       <c r="C6" s="3">
@@ -6050,7 +6062,7 @@
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="B7">
         <v>5</v>
       </c>
       <c r="C7" s="3">
@@ -6073,7 +6085,7 @@
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="B8">
         <v>6</v>
       </c>
       <c r="C8" s="3">
@@ -6093,7 +6105,7 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="B9">
         <v>7</v>
       </c>
       <c r="C9" s="3">
@@ -6113,7 +6125,7 @@
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="B10">
         <v>8</v>
       </c>
       <c r="C10" s="3">
@@ -6136,7 +6148,7 @@
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="3">
@@ -6159,7 +6171,7 @@
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="B12">
         <v>9</v>
       </c>
       <c r="C12" s="2">
@@ -6182,7 +6194,7 @@
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="B13">
         <v>10</v>
       </c>
       <c r="K13" t="s">
@@ -6193,7 +6205,7 @@
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="B14">
         <v>11</v>
       </c>
       <c r="L14" t="s">
@@ -6207,7 +6219,7 @@
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="B15">
         <v>12</v>
       </c>
       <c r="C15" s="2">
@@ -6233,7 +6245,7 @@
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="B16">
         <v>13</v>
       </c>
       <c r="Q16" t="s">
@@ -6243,8 +6255,8 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A17">
+    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B17">
         <v>14</v>
       </c>
       <c r="C17" s="2">
@@ -6263,16 +6275,16 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A18">
+    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B18">
         <v>15</v>
       </c>
       <c r="R18" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19">
+    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B19">
         <v>16</v>
       </c>
       <c r="F19">
@@ -6285,16 +6297,16 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20">
+    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B20">
         <v>17</v>
       </c>
       <c r="R20" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21">
+    <row r="21" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B21">
         <v>18</v>
       </c>
       <c r="F21">
@@ -6310,8 +6322,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22">
+    <row r="22" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B22">
         <v>19</v>
       </c>
       <c r="F22">
@@ -6324,8 +6336,8 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23">
+    <row r="23" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B23">
         <v>20</v>
       </c>
       <c r="C23">
@@ -6347,8 +6359,8 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24">
+    <row r="24" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B24">
         <v>21</v>
       </c>
       <c r="C24" s="2">
@@ -6370,8 +6382,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25">
+    <row r="25" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B25">
         <v>22</v>
       </c>
       <c r="C25" s="2">
@@ -6393,8 +6405,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26">
+    <row r="26" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B26">
         <v>23</v>
       </c>
       <c r="M26">
@@ -6407,8 +6419,8 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27">
+    <row r="27" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B27">
         <v>24</v>
       </c>
       <c r="C27">
@@ -6427,8 +6439,8 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28">
+    <row r="28" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B28">
         <v>25</v>
       </c>
       <c r="C28">
@@ -6444,8 +6456,8 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29">
+    <row r="29" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B29">
         <v>26</v>
       </c>
       <c r="F29">
@@ -6458,8 +6470,8 @@
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30">
+    <row r="30" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B30">
         <v>27</v>
       </c>
       <c r="C30">
@@ -6478,8 +6490,8 @@
         <v>68</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31">
+    <row r="31" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B31">
         <v>28</v>
       </c>
       <c r="C31">
@@ -6498,8 +6510,8 @@
         <v>522</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A32">
+    <row r="32" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B32">
         <v>29</v>
       </c>
       <c r="Q32">
@@ -6509,8 +6521,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A33">
+    <row r="33" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B33">
         <v>30</v>
       </c>
       <c r="C33">
@@ -6529,8 +6541,8 @@
         <v>563</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A34">
+    <row r="34" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B34">
         <v>31</v>
       </c>
       <c r="C34">
@@ -6552,8 +6564,8 @@
         <v>461</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A35">
+    <row r="35" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B35">
         <v>32</v>
       </c>
       <c r="C35">
@@ -6572,8 +6584,8 @@
         <v>482</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A36">
+    <row r="36" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B36">
         <v>33</v>
       </c>
       <c r="F36">
@@ -6586,8 +6598,8 @@
         <v>586</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A37">
+    <row r="37" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B37">
         <v>34</v>
       </c>
       <c r="F37">
@@ -6597,7 +6609,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:18" x14ac:dyDescent="0.25">
       <c r="O38">
         <v>0</v>
       </c>
@@ -6605,8 +6617,8 @@
         <v>657</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A39">
+    <row r="39" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B39">
         <v>35</v>
       </c>
       <c r="C39">
@@ -6634,8 +6646,8 @@
         <v>662</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A40">
+    <row r="40" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B40">
         <v>36</v>
       </c>
       <c r="C40">
@@ -6657,8 +6669,8 @@
         <v>666</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A41">
+    <row r="41" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B41">
         <v>37</v>
       </c>
       <c r="M41">
@@ -6671,8 +6683,8 @@
         <v>668</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A42">
+    <row r="42" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B42">
         <v>38</v>
       </c>
       <c r="C42">
@@ -6697,8 +6709,8 @@
         <v>671</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A43">
+    <row r="43" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B43">
         <v>39</v>
       </c>
       <c r="C43">
@@ -6723,8 +6735,8 @@
         <v>975</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A44">
+    <row r="44" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B44">
         <v>40</v>
       </c>
       <c r="C44">
@@ -6746,8 +6758,8 @@
         <v>673</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A45">
+    <row r="45" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B45">
         <v>41</v>
       </c>
       <c r="C45">
@@ -6766,8 +6778,8 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A46">
+    <row r="46" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B46">
         <v>42</v>
       </c>
       <c r="C46">
@@ -6786,8 +6798,8 @@
         <v>999</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A47">
+    <row r="47" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B47">
         <v>43</v>
       </c>
       <c r="C47">
@@ -6806,7 +6818,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C48">
         <v>-0.59913658322029595</v>
       </c>
@@ -7164,12 +7176,12 @@
       </c>
     </row>
     <row r="69" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="25"/>
+      <c r="A69" s="25"/>
       <c r="P69" s="25"/>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="23" t="s">
-        <v>742</v>
+      <c r="A70" s="23" t="s">
+        <v>741</v>
       </c>
       <c r="C70">
         <v>-1.2038</v>
@@ -7245,7 +7257,7 @@
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A74">
+      <c r="B74">
         <v>4</v>
       </c>
       <c r="C74">
@@ -7265,7 +7277,7 @@
       </c>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A75">
+      <c r="B75">
         <v>5</v>
       </c>
       <c r="C75">
@@ -7288,7 +7300,7 @@
       </c>
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A76">
+      <c r="B76">
         <v>6</v>
       </c>
       <c r="C76" s="23">
@@ -7311,10 +7323,10 @@
       </c>
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A77" s="22" t="s">
+      <c r="A77" s="22"/>
+      <c r="B77" s="22" t="s">
         <v>721</v>
       </c>
-      <c r="B77" s="22"/>
       <c r="F77">
         <v>0.7</v>
       </c>
@@ -7323,7 +7335,7 @@
       </c>
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A78">
+      <c r="B78">
         <v>7</v>
       </c>
       <c r="F78">
@@ -7352,7 +7364,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:19" x14ac:dyDescent="0.25">
       <c r="I81">
         <v>0.9</v>
       </c>
@@ -7363,12 +7375,12 @@
         <v>722</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:19" x14ac:dyDescent="0.25">
       <c r="R82" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:19" x14ac:dyDescent="0.25">
       <c r="G83">
         <v>0.9</v>
       </c>
@@ -7376,7 +7388,7 @@
         <v>1311</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:19" x14ac:dyDescent="0.25">
       <c r="I84">
         <v>0.85</v>
       </c>
@@ -7384,7 +7396,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:19" x14ac:dyDescent="0.25">
       <c r="F85">
         <v>0.7</v>
       </c>
@@ -7392,7 +7404,7 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:19" x14ac:dyDescent="0.25">
       <c r="I86">
         <v>0.8</v>
       </c>
@@ -7400,7 +7412,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:19" x14ac:dyDescent="0.25">
       <c r="I87">
         <v>0.75</v>
       </c>
@@ -7408,8 +7420,8 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A88">
+    <row r="88" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B88">
         <v>18</v>
       </c>
       <c r="G88">
@@ -7425,8 +7437,8 @@
         <v>724</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A89">
+    <row r="89" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B89">
         <v>19</v>
       </c>
       <c r="Q89">
@@ -7436,8 +7448,8 @@
         <v>725</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A90">
+    <row r="90" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B90">
         <v>20</v>
       </c>
       <c r="F90">
@@ -7447,8 +7459,8 @@
         <v>1939</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A91">
+    <row r="91" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B91">
         <v>21</v>
       </c>
       <c r="G91">
@@ -7461,8 +7473,8 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A92">
+    <row r="92" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B92">
         <v>22</v>
       </c>
       <c r="F92">
@@ -7475,8 +7487,8 @@
         <v>726</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A93">
+    <row r="93" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B93">
         <v>23</v>
       </c>
       <c r="H93">
@@ -7486,8 +7498,8 @@
         <v>1399</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A94">
+    <row r="94" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B94">
         <v>24</v>
       </c>
       <c r="F94">
@@ -7497,8 +7509,8 @@
         <v>1256</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A95">
+    <row r="95" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B95">
         <v>25</v>
       </c>
       <c r="F95">
@@ -7508,8 +7520,8 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A96">
+    <row r="96" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B96">
         <v>26</v>
       </c>
       <c r="F96">
@@ -7533,7 +7545,7 @@
       </c>
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A99">
+      <c r="B99">
         <v>29</v>
       </c>
       <c r="P99" s="23" t="s">
@@ -7544,7 +7556,7 @@
       </c>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A100">
+      <c r="B100">
         <v>30</v>
       </c>
       <c r="F100">
@@ -7555,7 +7567,7 @@
       </c>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A101">
+      <c r="B101">
         <v>31</v>
       </c>
       <c r="I101">
@@ -7566,11 +7578,11 @@
       </c>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A102">
+      <c r="A102" s="23" t="s">
+        <v>740</v>
+      </c>
+      <c r="B102">
         <v>1</v>
-      </c>
-      <c r="B102" s="23" t="s">
-        <v>741</v>
       </c>
       <c r="Q102">
         <v>2033</v>
@@ -7583,11 +7595,11 @@
       </c>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A103">
+      <c r="A103" s="23" t="s">
+        <v>741</v>
+      </c>
+      <c r="B103">
         <v>32</v>
-      </c>
-      <c r="B103" s="23" t="s">
-        <v>742</v>
       </c>
       <c r="F103">
         <v>0.8</v>
@@ -7597,11 +7609,11 @@
       </c>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A104">
+      <c r="A104" s="23" t="s">
+        <v>740</v>
+      </c>
+      <c r="B104">
         <v>2</v>
-      </c>
-      <c r="B104" s="23" t="s">
-        <v>741</v>
       </c>
       <c r="Q104">
         <v>1322</v>
@@ -7611,11 +7623,11 @@
       </c>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A105">
+      <c r="A105" s="23" t="s">
+        <v>741</v>
+      </c>
+      <c r="B105">
         <v>33</v>
-      </c>
-      <c r="B105" s="23" t="s">
-        <v>742</v>
       </c>
       <c r="F105">
         <v>1</v>
@@ -7631,11 +7643,11 @@
       </c>
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A106">
+      <c r="A106" s="23" t="s">
+        <v>741</v>
+      </c>
+      <c r="B106">
         <v>34</v>
-      </c>
-      <c r="B106" s="23" t="s">
-        <v>742</v>
       </c>
       <c r="Q106">
         <v>938</v>
@@ -7648,11 +7660,11 @@
       </c>
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A107">
+      <c r="A107" s="23" t="s">
+        <v>741</v>
+      </c>
+      <c r="B107">
         <v>35</v>
-      </c>
-      <c r="B107" s="23" t="s">
-        <v>742</v>
       </c>
       <c r="Q107">
         <v>925</v>
@@ -7662,11 +7674,11 @@
       </c>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A108">
+      <c r="A108" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="B108">
         <v>2</v>
-      </c>
-      <c r="B108" s="23" t="s">
-        <v>743</v>
       </c>
       <c r="Q108">
         <v>943</v>
@@ -7676,7 +7688,7 @@
       </c>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A110">
+      <c r="B110">
         <v>4</v>
       </c>
       <c r="Q110">
@@ -7687,7 +7699,7 @@
       </c>
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A111">
+      <c r="B111">
         <v>5</v>
       </c>
       <c r="Q111">
@@ -7695,6 +7707,54 @@
       </c>
       <c r="R111" t="s">
         <v>745</v>
+      </c>
+      <c r="S111" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A112" s="23" t="s">
+        <v>743</v>
+      </c>
+      <c r="B112">
+        <v>1</v>
+      </c>
+      <c r="Q112">
+        <v>0.04</v>
+      </c>
+      <c r="R112" t="s">
+        <v>746</v>
+      </c>
+      <c r="S112" s="23" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A113" s="23" t="s">
+        <v>742</v>
+      </c>
+      <c r="B113">
+        <v>9</v>
+      </c>
+      <c r="C113">
+        <v>-3.1486202185996501</v>
+      </c>
+      <c r="D113">
+        <v>1.26914376889979</v>
+      </c>
+      <c r="E113">
+        <v>-4.8520029130770999</v>
+      </c>
+      <c r="Q113">
+        <v>5.5E-2</v>
+      </c>
+      <c r="R113" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A114" s="23" t="s">
+        <v>743</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
multiple updates, both 0D and 1D running
</commit_message>
<xml_diff>
--- a/aysha/FittingTests v3.xlsx
+++ b/aysha/FittingTests v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\kkakosim\github\tamuq-chen-secarelab-receiver\aysha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B23D3CE-AE50-4D97-AFC6-605C5039AEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B5C9CF-77D3-496F-AD82-76D6606927CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="752">
   <si>
     <t>A</t>
   </si>
@@ -2382,6 +2382,12 @@
   </si>
   <si>
     <t>model</t>
+  </si>
+  <si>
+    <t>3 stages optimi\tion (heating, cooling, heating)</t>
+  </si>
+  <si>
+    <t>solid scatter plot, good but gas not</t>
   </si>
 </sst>
 </file>
@@ -5880,7 +5886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:S114"/>
+  <dimension ref="A2:S116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="23"/>
@@ -7729,7 +7735,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A113" s="23" t="s">
         <v>742</v>
       </c>
@@ -7752,9 +7758,34 @@
         <v>748</v>
       </c>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A114" s="23" t="s">
         <v>743</v>
+      </c>
+      <c r="B114">
+        <v>3</v>
+      </c>
+      <c r="Q114">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B115">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B116">
+        <v>6</v>
+      </c>
+      <c r="Q116">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="R116" t="s">
+        <v>750</v>
+      </c>
+      <c r="S116" t="s">
+        <v>751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
attempting to introduce the proper flow obstruction
</commit_message>
<xml_diff>
--- a/aysha/FittingTests v3.xlsx
+++ b/aysha/FittingTests v3.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\kkakosim\github\tamuq-chen-secarelab-receiver\aysha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{F9B05BD3-6F93-43EB-89E4-4E1E10B2B816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E2D2087-D4D8-42D0-BFB2-EAFB2FDD3BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0D" sheetId="1" r:id="rId1"/>
     <sheet name="3D" sheetId="2" r:id="rId2"/>
     <sheet name="Optical" sheetId="3" r:id="rId3"/>
+    <sheet name="MFC_t0" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="831">
   <si>
     <t>A</t>
   </si>
@@ -2398,6 +2398,234 @@
   </si>
   <si>
     <t xml:space="preserve">tested </t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Clock Time</t>
+  </si>
+  <si>
+    <t>Time (s)</t>
+  </si>
+  <si>
+    <t>MFC H2 SP (lpm)</t>
+  </si>
+  <si>
+    <t>MFC CH4 SP (lpm)</t>
+  </si>
+  <si>
+    <t>MFC CO2 SP (lpm)</t>
+  </si>
+  <si>
+    <t>MFC He SP (lpm)</t>
+  </si>
+  <si>
+    <t>MFC H2 (lpm)</t>
+  </si>
+  <si>
+    <t>MFC CH4 (lpm)</t>
+  </si>
+  <si>
+    <t>MFC CO2 (lpm)</t>
+  </si>
+  <si>
+    <t>MFC He (lpm)</t>
+  </si>
+  <si>
+    <t>P1 Limit (mbarg)</t>
+  </si>
+  <si>
+    <t>P2 Limit (mbarg)</t>
+  </si>
+  <si>
+    <t>DP1 Limit (mbar)</t>
+  </si>
+  <si>
+    <t>DP2 Limit (mbar)</t>
+  </si>
+  <si>
+    <t>P1 (mbarg)</t>
+  </si>
+  <si>
+    <t>P2 (mbarg)</t>
+  </si>
+  <si>
+    <t>DP1 (mbar)</t>
+  </si>
+  <si>
+    <t>DP2 (mbar)</t>
+  </si>
+  <si>
+    <t>T1 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T2 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T3 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T4 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T5 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T6 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T7 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T8 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T9 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T10 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T11 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T12 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T13 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T14 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T15 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T16 Limit (°C)</t>
+  </si>
+  <si>
+    <t>T1 (°C)</t>
+  </si>
+  <si>
+    <t>T2 (°C)</t>
+  </si>
+  <si>
+    <t>T3 (°C)</t>
+  </si>
+  <si>
+    <t>T4 (°C)</t>
+  </si>
+  <si>
+    <t>T5 (°C)</t>
+  </si>
+  <si>
+    <t>T6 (°C)</t>
+  </si>
+  <si>
+    <t>T7 (°C)</t>
+  </si>
+  <si>
+    <t>T8 (°C)</t>
+  </si>
+  <si>
+    <t>T09 (°C)</t>
+  </si>
+  <si>
+    <t>T10 (°C)</t>
+  </si>
+  <si>
+    <t>T11 (°C)</t>
+  </si>
+  <si>
+    <t>T12 (°C)</t>
+  </si>
+  <si>
+    <t>T13 (°C)</t>
+  </si>
+  <si>
+    <t>T14 (°C)</t>
+  </si>
+  <si>
+    <t>T15 (°C)</t>
+  </si>
+  <si>
+    <t>T16 (°C)</t>
+  </si>
+  <si>
+    <t>Flow Module</t>
+  </si>
+  <si>
+    <t>Pressure Module</t>
+  </si>
+  <si>
+    <t>Temperature Module</t>
+  </si>
+  <si>
+    <t>Program Started</t>
+  </si>
+  <si>
+    <t>MFCs Manual</t>
+  </si>
+  <si>
+    <t>Alarm Triggered</t>
+  </si>
+  <si>
+    <t>Overpressure</t>
+  </si>
+  <si>
+    <t>Overtemperature</t>
+  </si>
+  <si>
+    <t>Emergency User Input</t>
+  </si>
+  <si>
+    <t>Flows Emergency Stop</t>
+  </si>
+  <si>
+    <t>Flow Module Comm Error</t>
+  </si>
+  <si>
+    <t>Pressure Module Comm Error</t>
+  </si>
+  <si>
+    <t>Temperature Module Comm Error</t>
+  </si>
+  <si>
+    <t>E69</t>
+  </si>
+  <si>
+    <t>E70</t>
+  </si>
+  <si>
+    <t>E71</t>
+  </si>
+  <si>
+    <t>E72</t>
+  </si>
+  <si>
+    <t>E73</t>
+  </si>
+  <si>
+    <t>E74</t>
+  </si>
+  <si>
+    <t>E75</t>
+  </si>
+  <si>
+    <t>E76</t>
+  </si>
+  <si>
+    <t>E77</t>
+  </si>
+  <si>
+    <t>E79</t>
+  </si>
+  <si>
+    <t>E80</t>
+  </si>
+  <si>
+    <t>E81</t>
   </si>
 </sst>
 </file>
@@ -2519,7 +2747,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2575,6 +2803,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4189,6 +4418,433 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="3.0665354330708661E-2"/>
+                  <c:y val="-4.2117964421114026E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>MFC_t0!$L$2:$L$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>15.273</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12.496</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.509</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9.097999999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7.104000000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>19.488</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13.169999999999998</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9.016</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6.9399999999999995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5149999999999997</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>13.844999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10.007000000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.0109999999999992</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5990000000000002</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.5110000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>MFC_t0!$S$2:$S$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>0.14299999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-7.1999999999999995E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-3.9E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.222</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.29499999999999998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.26600000000000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.23300000000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.29899999999999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-0.38700000000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>6.2E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-0.13900000000000001</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-0.22600000000000001</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.29899999999999999</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-0.36799999999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C448-4EFE-96A5-25781AA5A6D9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2130121920"/>
+        <c:axId val="2130123360"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="2130121920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2130123360"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2130123360"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2130121920"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -4230,6 +4886,46 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5301,6 +5997,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -5575,6 +6787,47 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>61912</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>138112</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C5FD98D-454C-CD33-865A-BE1644303320}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -12353,4 +13606,3179 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8FCA6E0-29A7-4D5D-82E5-A39A92764F1E}">
+  <dimension ref="A1:BM16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>755</v>
+      </c>
+      <c r="B1" t="s">
+        <v>756</v>
+      </c>
+      <c r="C1" t="s">
+        <v>757</v>
+      </c>
+      <c r="D1" t="s">
+        <v>758</v>
+      </c>
+      <c r="E1" t="s">
+        <v>759</v>
+      </c>
+      <c r="F1" t="s">
+        <v>760</v>
+      </c>
+      <c r="G1" t="s">
+        <v>761</v>
+      </c>
+      <c r="H1" t="s">
+        <v>762</v>
+      </c>
+      <c r="I1" t="s">
+        <v>763</v>
+      </c>
+      <c r="J1" t="s">
+        <v>764</v>
+      </c>
+      <c r="K1" t="s">
+        <v>765</v>
+      </c>
+      <c r="M1" t="s">
+        <v>766</v>
+      </c>
+      <c r="N1" t="s">
+        <v>767</v>
+      </c>
+      <c r="O1" t="s">
+        <v>768</v>
+      </c>
+      <c r="P1" t="s">
+        <v>769</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>770</v>
+      </c>
+      <c r="R1" t="s">
+        <v>771</v>
+      </c>
+      <c r="S1" t="s">
+        <v>772</v>
+      </c>
+      <c r="T1" t="s">
+        <v>773</v>
+      </c>
+      <c r="U1" t="s">
+        <v>774</v>
+      </c>
+      <c r="V1" t="s">
+        <v>775</v>
+      </c>
+      <c r="W1" t="s">
+        <v>776</v>
+      </c>
+      <c r="X1" t="s">
+        <v>777</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>778</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>779</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>780</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>781</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>782</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>783</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>784</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>785</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>786</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>787</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>788</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>789</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>790</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>791</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>792</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>793</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>794</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>795</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>796</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>797</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>798</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>799</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>800</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>801</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>802</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>803</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>804</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>805</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>806</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>807</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>808</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>809</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>810</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>811</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>812</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>813</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>814</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>815</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>816</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>817</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="2" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B2" s="23">
+        <v>0.67929398148148146</v>
+      </c>
+      <c r="C2">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>3.7</v>
+      </c>
+      <c r="E2">
+        <v>3.7</v>
+      </c>
+      <c r="F2">
+        <v>3.7</v>
+      </c>
+      <c r="G2">
+        <v>1.7</v>
+      </c>
+      <c r="H2">
+        <v>3.669</v>
+      </c>
+      <c r="I2">
+        <v>5.2889999999999997</v>
+      </c>
+      <c r="J2">
+        <v>5.1429999999999998</v>
+      </c>
+      <c r="K2">
+        <v>1.1719999999999999</v>
+      </c>
+      <c r="L2">
+        <f>SUM(H2:K2)</f>
+        <v>15.273</v>
+      </c>
+      <c r="M2">
+        <v>500</v>
+      </c>
+      <c r="N2">
+        <v>200</v>
+      </c>
+      <c r="O2">
+        <v>200</v>
+      </c>
+      <c r="P2">
+        <v>100</v>
+      </c>
+      <c r="Q2">
+        <v>0.67200000000000004</v>
+      </c>
+      <c r="R2">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="S2">
+        <v>0.14299999999999999</v>
+      </c>
+      <c r="T2">
+        <v>-0.28899999999999998</v>
+      </c>
+      <c r="U2">
+        <v>1500</v>
+      </c>
+      <c r="V2">
+        <v>1500</v>
+      </c>
+      <c r="W2">
+        <v>1500</v>
+      </c>
+      <c r="X2">
+        <v>1500</v>
+      </c>
+      <c r="Y2">
+        <v>1500</v>
+      </c>
+      <c r="Z2">
+        <v>1500</v>
+      </c>
+      <c r="AA2">
+        <v>1500</v>
+      </c>
+      <c r="AB2">
+        <v>1500</v>
+      </c>
+      <c r="AC2">
+        <v>1500</v>
+      </c>
+      <c r="AD2">
+        <v>1500</v>
+      </c>
+      <c r="AE2">
+        <v>1500</v>
+      </c>
+      <c r="AF2">
+        <v>1500</v>
+      </c>
+      <c r="AG2">
+        <v>1500</v>
+      </c>
+      <c r="AH2">
+        <v>1500</v>
+      </c>
+      <c r="AI2">
+        <v>1500</v>
+      </c>
+      <c r="AJ2">
+        <v>1500</v>
+      </c>
+      <c r="AK2">
+        <v>22.277999999999999</v>
+      </c>
+      <c r="AL2">
+        <v>20.251999999999999</v>
+      </c>
+      <c r="AM2">
+        <v>23.46</v>
+      </c>
+      <c r="AN2">
+        <v>22.001999999999999</v>
+      </c>
+      <c r="AO2">
+        <v>18.645</v>
+      </c>
+      <c r="AP2">
+        <v>25.114000000000001</v>
+      </c>
+      <c r="AQ2">
+        <v>24.907</v>
+      </c>
+      <c r="AR2">
+        <v>23.423999999999999</v>
+      </c>
+      <c r="AS2">
+        <v>23.01</v>
+      </c>
+      <c r="AT2">
+        <v>23.207000000000001</v>
+      </c>
+      <c r="AU2">
+        <v>23.143000000000001</v>
+      </c>
+      <c r="AV2">
+        <v>23.05</v>
+      </c>
+      <c r="AW2">
+        <v>20.27</v>
+      </c>
+      <c r="AX2">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="AY2">
+        <v>20.289000000000001</v>
+      </c>
+      <c r="AZ2">
+        <v>20.157</v>
+      </c>
+      <c r="BA2">
+        <v>1</v>
+      </c>
+      <c r="BB2">
+        <v>1</v>
+      </c>
+      <c r="BC2">
+        <v>1</v>
+      </c>
+      <c r="BD2">
+        <v>0</v>
+      </c>
+      <c r="BE2">
+        <v>1</v>
+      </c>
+      <c r="BF2">
+        <v>0</v>
+      </c>
+      <c r="BG2">
+        <v>0</v>
+      </c>
+      <c r="BH2">
+        <v>0</v>
+      </c>
+      <c r="BI2">
+        <v>0</v>
+      </c>
+      <c r="BJ2">
+        <v>0</v>
+      </c>
+      <c r="BK2">
+        <v>0</v>
+      </c>
+      <c r="BL2">
+        <v>0</v>
+      </c>
+      <c r="BM2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>485</v>
+      </c>
+      <c r="B3" s="23">
+        <v>0.49829861111111112</v>
+      </c>
+      <c r="C3">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>3.7</v>
+      </c>
+      <c r="E3">
+        <v>3.7</v>
+      </c>
+      <c r="F3">
+        <v>1.7</v>
+      </c>
+      <c r="G3">
+        <v>1.7</v>
+      </c>
+      <c r="H3">
+        <v>3.665</v>
+      </c>
+      <c r="I3">
+        <v>5.2939999999999996</v>
+      </c>
+      <c r="J3">
+        <v>2.3639999999999999</v>
+      </c>
+      <c r="K3">
+        <v>1.173</v>
+      </c>
+      <c r="L3">
+        <f t="shared" ref="L3:L16" si="0">SUM(H3:K3)</f>
+        <v>12.496</v>
+      </c>
+      <c r="M3">
+        <v>500</v>
+      </c>
+      <c r="N3">
+        <v>200</v>
+      </c>
+      <c r="O3">
+        <v>200</v>
+      </c>
+      <c r="P3">
+        <v>100</v>
+      </c>
+      <c r="Q3">
+        <v>0.67800000000000005</v>
+      </c>
+      <c r="R3">
+        <v>0.40200000000000002</v>
+      </c>
+      <c r="S3">
+        <v>-7.1999999999999995E-2</v>
+      </c>
+      <c r="T3">
+        <v>-0.313</v>
+      </c>
+      <c r="U3">
+        <v>1500</v>
+      </c>
+      <c r="V3">
+        <v>1500</v>
+      </c>
+      <c r="W3">
+        <v>1500</v>
+      </c>
+      <c r="X3">
+        <v>1500</v>
+      </c>
+      <c r="Y3">
+        <v>1500</v>
+      </c>
+      <c r="Z3">
+        <v>1500</v>
+      </c>
+      <c r="AA3">
+        <v>1500</v>
+      </c>
+      <c r="AB3">
+        <v>1500</v>
+      </c>
+      <c r="AC3">
+        <v>1500</v>
+      </c>
+      <c r="AD3">
+        <v>1500</v>
+      </c>
+      <c r="AE3">
+        <v>1500</v>
+      </c>
+      <c r="AF3">
+        <v>1500</v>
+      </c>
+      <c r="AG3">
+        <v>1500</v>
+      </c>
+      <c r="AH3">
+        <v>1500</v>
+      </c>
+      <c r="AI3">
+        <v>1500</v>
+      </c>
+      <c r="AJ3">
+        <v>1500</v>
+      </c>
+      <c r="AK3">
+        <v>20.167999999999999</v>
+      </c>
+      <c r="AL3">
+        <v>20.321999999999999</v>
+      </c>
+      <c r="AM3">
+        <v>20.523</v>
+      </c>
+      <c r="AN3">
+        <v>20.370999999999999</v>
+      </c>
+      <c r="AO3">
+        <v>18.364000000000001</v>
+      </c>
+      <c r="AP3">
+        <v>25.265000000000001</v>
+      </c>
+      <c r="AQ3">
+        <v>25.013999999999999</v>
+      </c>
+      <c r="AR3">
+        <v>21.701000000000001</v>
+      </c>
+      <c r="AS3">
+        <v>20.433</v>
+      </c>
+      <c r="AT3">
+        <v>20.498999999999999</v>
+      </c>
+      <c r="AU3">
+        <v>20.335999999999999</v>
+      </c>
+      <c r="AV3">
+        <v>20.420999999999999</v>
+      </c>
+      <c r="AW3">
+        <v>20.341999999999999</v>
+      </c>
+      <c r="AX3">
+        <v>20.135999999999999</v>
+      </c>
+      <c r="AY3">
+        <v>20.353000000000002</v>
+      </c>
+      <c r="AZ3">
+        <v>20.222999999999999</v>
+      </c>
+      <c r="BA3">
+        <v>1</v>
+      </c>
+      <c r="BB3">
+        <v>1</v>
+      </c>
+      <c r="BC3">
+        <v>1</v>
+      </c>
+      <c r="BD3">
+        <v>0</v>
+      </c>
+      <c r="BE3">
+        <v>1</v>
+      </c>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3">
+        <v>0</v>
+      </c>
+      <c r="BH3">
+        <v>0</v>
+      </c>
+      <c r="BI3">
+        <v>0</v>
+      </c>
+      <c r="BJ3">
+        <v>0</v>
+      </c>
+      <c r="BK3">
+        <v>0</v>
+      </c>
+      <c r="BL3">
+        <v>0</v>
+      </c>
+      <c r="BM3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>819</v>
+      </c>
+      <c r="B4" s="23">
+        <v>0.5847106481481481</v>
+      </c>
+      <c r="C4">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>3.7</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>1.7</v>
+      </c>
+      <c r="H4">
+        <v>3.67</v>
+      </c>
+      <c r="I4">
+        <v>2.8690000000000002</v>
+      </c>
+      <c r="J4">
+        <v>2.794</v>
+      </c>
+      <c r="K4">
+        <v>1.1759999999999999</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="0"/>
+        <v>10.509</v>
+      </c>
+      <c r="M4">
+        <v>500</v>
+      </c>
+      <c r="N4">
+        <v>200</v>
+      </c>
+      <c r="O4">
+        <v>200</v>
+      </c>
+      <c r="P4">
+        <v>100</v>
+      </c>
+      <c r="Q4">
+        <v>0.69</v>
+      </c>
+      <c r="R4">
+        <v>0.38300000000000001</v>
+      </c>
+      <c r="S4">
+        <v>-3.9E-2</v>
+      </c>
+      <c r="T4">
+        <v>-0.27600000000000002</v>
+      </c>
+      <c r="U4">
+        <v>1500</v>
+      </c>
+      <c r="V4">
+        <v>1500</v>
+      </c>
+      <c r="W4">
+        <v>1500</v>
+      </c>
+      <c r="X4">
+        <v>1500</v>
+      </c>
+      <c r="Y4">
+        <v>1500</v>
+      </c>
+      <c r="Z4">
+        <v>1500</v>
+      </c>
+      <c r="AA4">
+        <v>1500</v>
+      </c>
+      <c r="AB4">
+        <v>1500</v>
+      </c>
+      <c r="AC4">
+        <v>1500</v>
+      </c>
+      <c r="AD4">
+        <v>1500</v>
+      </c>
+      <c r="AE4">
+        <v>1500</v>
+      </c>
+      <c r="AF4">
+        <v>1500</v>
+      </c>
+      <c r="AG4">
+        <v>1500</v>
+      </c>
+      <c r="AH4">
+        <v>1500</v>
+      </c>
+      <c r="AI4">
+        <v>1500</v>
+      </c>
+      <c r="AJ4">
+        <v>1500</v>
+      </c>
+      <c r="AK4">
+        <v>59.156999999999996</v>
+      </c>
+      <c r="AL4">
+        <v>53.396999999999998</v>
+      </c>
+      <c r="AM4">
+        <v>107.42100000000001</v>
+      </c>
+      <c r="AN4">
+        <v>38.183999999999997</v>
+      </c>
+      <c r="AO4">
+        <v>23.056000000000001</v>
+      </c>
+      <c r="AP4">
+        <v>25.128</v>
+      </c>
+      <c r="AQ4">
+        <v>24.975000000000001</v>
+      </c>
+      <c r="AR4">
+        <v>44.439</v>
+      </c>
+      <c r="AS4">
+        <v>71.262</v>
+      </c>
+      <c r="AT4">
+        <v>98.691000000000003</v>
+      </c>
+      <c r="AU4">
+        <v>87.981999999999999</v>
+      </c>
+      <c r="AV4">
+        <v>64.507000000000005</v>
+      </c>
+      <c r="AW4">
+        <v>24.576000000000001</v>
+      </c>
+      <c r="AX4">
+        <v>24.337</v>
+      </c>
+      <c r="AY4">
+        <v>24.14</v>
+      </c>
+      <c r="AZ4">
+        <v>24.15</v>
+      </c>
+      <c r="BA4">
+        <v>1</v>
+      </c>
+      <c r="BB4">
+        <v>1</v>
+      </c>
+      <c r="BC4">
+        <v>1</v>
+      </c>
+      <c r="BD4">
+        <v>0</v>
+      </c>
+      <c r="BE4">
+        <v>1</v>
+      </c>
+      <c r="BF4">
+        <v>0</v>
+      </c>
+      <c r="BG4">
+        <v>0</v>
+      </c>
+      <c r="BH4">
+        <v>0</v>
+      </c>
+      <c r="BI4">
+        <v>0</v>
+      </c>
+      <c r="BJ4">
+        <v>0</v>
+      </c>
+      <c r="BK4">
+        <v>0</v>
+      </c>
+      <c r="BL4">
+        <v>0</v>
+      </c>
+      <c r="BM4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>820</v>
+      </c>
+      <c r="B5" s="23">
+        <v>0.37761574074074072</v>
+      </c>
+      <c r="C5">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>3.7</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1.7</v>
+      </c>
+      <c r="H5">
+        <v>3.6640000000000001</v>
+      </c>
+      <c r="I5">
+        <v>2.8650000000000002</v>
+      </c>
+      <c r="J5">
+        <v>1.3979999999999999</v>
+      </c>
+      <c r="K5">
+        <v>1.171</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="0"/>
+        <v>9.097999999999999</v>
+      </c>
+      <c r="M5">
+        <v>500</v>
+      </c>
+      <c r="N5">
+        <v>200</v>
+      </c>
+      <c r="O5">
+        <v>200</v>
+      </c>
+      <c r="P5">
+        <v>100</v>
+      </c>
+      <c r="Q5">
+        <v>0.68200000000000005</v>
+      </c>
+      <c r="R5">
+        <v>0.40500000000000003</v>
+      </c>
+      <c r="S5">
+        <v>-0.222</v>
+      </c>
+      <c r="T5">
+        <v>-0.309</v>
+      </c>
+      <c r="U5">
+        <v>1500</v>
+      </c>
+      <c r="V5">
+        <v>1500</v>
+      </c>
+      <c r="W5">
+        <v>1500</v>
+      </c>
+      <c r="X5">
+        <v>1500</v>
+      </c>
+      <c r="Y5">
+        <v>1500</v>
+      </c>
+      <c r="Z5">
+        <v>1500</v>
+      </c>
+      <c r="AA5">
+        <v>1500</v>
+      </c>
+      <c r="AB5">
+        <v>1500</v>
+      </c>
+      <c r="AC5">
+        <v>1500</v>
+      </c>
+      <c r="AD5">
+        <v>1500</v>
+      </c>
+      <c r="AE5">
+        <v>1500</v>
+      </c>
+      <c r="AF5">
+        <v>1500</v>
+      </c>
+      <c r="AG5">
+        <v>1500</v>
+      </c>
+      <c r="AH5">
+        <v>1500</v>
+      </c>
+      <c r="AI5">
+        <v>1500</v>
+      </c>
+      <c r="AJ5">
+        <v>1500</v>
+      </c>
+      <c r="AK5">
+        <v>20.518000000000001</v>
+      </c>
+      <c r="AL5">
+        <v>20.356000000000002</v>
+      </c>
+      <c r="AM5">
+        <v>20.603999999999999</v>
+      </c>
+      <c r="AN5">
+        <v>20.399000000000001</v>
+      </c>
+      <c r="AO5">
+        <v>18.347999999999999</v>
+      </c>
+      <c r="AP5">
+        <v>24.672999999999998</v>
+      </c>
+      <c r="AQ5">
+        <v>24.448</v>
+      </c>
+      <c r="AR5">
+        <v>21.797999999999998</v>
+      </c>
+      <c r="AS5">
+        <v>20.5</v>
+      </c>
+      <c r="AT5">
+        <v>20.605</v>
+      </c>
+      <c r="AU5">
+        <v>20.408000000000001</v>
+      </c>
+      <c r="AV5">
+        <v>20.515999999999998</v>
+      </c>
+      <c r="AW5">
+        <v>20.355</v>
+      </c>
+      <c r="AX5">
+        <v>20.138999999999999</v>
+      </c>
+      <c r="AY5">
+        <v>20.420000000000002</v>
+      </c>
+      <c r="AZ5">
+        <v>20.266999999999999</v>
+      </c>
+      <c r="BA5">
+        <v>1</v>
+      </c>
+      <c r="BB5">
+        <v>1</v>
+      </c>
+      <c r="BC5">
+        <v>1</v>
+      </c>
+      <c r="BD5">
+        <v>0</v>
+      </c>
+      <c r="BE5">
+        <v>1</v>
+      </c>
+      <c r="BF5">
+        <v>0</v>
+      </c>
+      <c r="BG5">
+        <v>0</v>
+      </c>
+      <c r="BH5">
+        <v>0</v>
+      </c>
+      <c r="BI5">
+        <v>0</v>
+      </c>
+      <c r="BJ5">
+        <v>0</v>
+      </c>
+      <c r="BK5">
+        <v>0</v>
+      </c>
+      <c r="BL5">
+        <v>0</v>
+      </c>
+      <c r="BM5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>821</v>
+      </c>
+      <c r="B6" s="23">
+        <v>0.43559027777777776</v>
+      </c>
+      <c r="C6">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>1.7</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1.7</v>
+      </c>
+      <c r="H6">
+        <v>1.6819999999999999</v>
+      </c>
+      <c r="I6">
+        <v>2.859</v>
+      </c>
+      <c r="J6">
+        <v>1.389</v>
+      </c>
+      <c r="K6">
+        <v>1.1739999999999999</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="0"/>
+        <v>7.104000000000001</v>
+      </c>
+      <c r="M6">
+        <v>500</v>
+      </c>
+      <c r="N6">
+        <v>200</v>
+      </c>
+      <c r="O6">
+        <v>200</v>
+      </c>
+      <c r="P6">
+        <v>100</v>
+      </c>
+      <c r="Q6">
+        <v>0.68</v>
+      </c>
+      <c r="R6">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="S6">
+        <v>-0.29499999999999998</v>
+      </c>
+      <c r="T6">
+        <v>-0.311</v>
+      </c>
+      <c r="U6">
+        <v>1500</v>
+      </c>
+      <c r="V6">
+        <v>1500</v>
+      </c>
+      <c r="W6">
+        <v>1500</v>
+      </c>
+      <c r="X6">
+        <v>1500</v>
+      </c>
+      <c r="Y6">
+        <v>1500</v>
+      </c>
+      <c r="Z6">
+        <v>1500</v>
+      </c>
+      <c r="AA6">
+        <v>1500</v>
+      </c>
+      <c r="AB6">
+        <v>1500</v>
+      </c>
+      <c r="AC6">
+        <v>1500</v>
+      </c>
+      <c r="AD6">
+        <v>1500</v>
+      </c>
+      <c r="AE6">
+        <v>1500</v>
+      </c>
+      <c r="AF6">
+        <v>1500</v>
+      </c>
+      <c r="AG6">
+        <v>1500</v>
+      </c>
+      <c r="AH6">
+        <v>1500</v>
+      </c>
+      <c r="AI6">
+        <v>1500</v>
+      </c>
+      <c r="AJ6">
+        <v>1500</v>
+      </c>
+      <c r="AK6">
+        <v>29.655999999999999</v>
+      </c>
+      <c r="AL6">
+        <v>20.463999999999999</v>
+      </c>
+      <c r="AM6">
+        <v>29.902999999999999</v>
+      </c>
+      <c r="AN6">
+        <v>21.088999999999999</v>
+      </c>
+      <c r="AO6">
+        <v>18.655000000000001</v>
+      </c>
+      <c r="AP6">
+        <v>25.138000000000002</v>
+      </c>
+      <c r="AQ6">
+        <v>24.934000000000001</v>
+      </c>
+      <c r="AR6">
+        <v>30.361000000000001</v>
+      </c>
+      <c r="AS6">
+        <v>33.777999999999999</v>
+      </c>
+      <c r="AT6">
+        <v>30.849</v>
+      </c>
+      <c r="AU6">
+        <v>32.182000000000002</v>
+      </c>
+      <c r="AV6">
+        <v>34.082999999999998</v>
+      </c>
+      <c r="AW6">
+        <v>20.681000000000001</v>
+      </c>
+      <c r="AX6">
+        <v>20.489000000000001</v>
+      </c>
+      <c r="AY6">
+        <v>20.672000000000001</v>
+      </c>
+      <c r="AZ6">
+        <v>20.545999999999999</v>
+      </c>
+      <c r="BA6">
+        <v>1</v>
+      </c>
+      <c r="BB6">
+        <v>1</v>
+      </c>
+      <c r="BC6">
+        <v>1</v>
+      </c>
+      <c r="BD6">
+        <v>0</v>
+      </c>
+      <c r="BE6">
+        <v>1</v>
+      </c>
+      <c r="BF6">
+        <v>0</v>
+      </c>
+      <c r="BG6">
+        <v>0</v>
+      </c>
+      <c r="BH6">
+        <v>0</v>
+      </c>
+      <c r="BI6">
+        <v>0</v>
+      </c>
+      <c r="BJ6">
+        <v>0</v>
+      </c>
+      <c r="BK6">
+        <v>0</v>
+      </c>
+      <c r="BL6">
+        <v>0</v>
+      </c>
+      <c r="BM6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>822</v>
+      </c>
+      <c r="B7" s="23">
+        <v>0.44568287037037035</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>4.4969999999999999</v>
+      </c>
+      <c r="I7">
+        <v>6.0190000000000001</v>
+      </c>
+      <c r="J7">
+        <v>5.524</v>
+      </c>
+      <c r="K7">
+        <v>3.448</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="0"/>
+        <v>19.488</v>
+      </c>
+      <c r="M7">
+        <v>500</v>
+      </c>
+      <c r="N7">
+        <v>200</v>
+      </c>
+      <c r="O7">
+        <v>200</v>
+      </c>
+      <c r="P7">
+        <v>100</v>
+      </c>
+      <c r="Q7">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="R7">
+        <v>0.40500000000000003</v>
+      </c>
+      <c r="S7">
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="T7">
+        <v>-0.29699999999999999</v>
+      </c>
+      <c r="U7">
+        <v>1500</v>
+      </c>
+      <c r="V7">
+        <v>1500</v>
+      </c>
+      <c r="W7">
+        <v>1500</v>
+      </c>
+      <c r="X7">
+        <v>1500</v>
+      </c>
+      <c r="Y7">
+        <v>1500</v>
+      </c>
+      <c r="Z7">
+        <v>1500</v>
+      </c>
+      <c r="AA7">
+        <v>1500</v>
+      </c>
+      <c r="AB7">
+        <v>1500</v>
+      </c>
+      <c r="AC7">
+        <v>1500</v>
+      </c>
+      <c r="AD7">
+        <v>1500</v>
+      </c>
+      <c r="AE7">
+        <v>1500</v>
+      </c>
+      <c r="AF7">
+        <v>1500</v>
+      </c>
+      <c r="AG7">
+        <v>1500</v>
+      </c>
+      <c r="AH7">
+        <v>1500</v>
+      </c>
+      <c r="AI7">
+        <v>1500</v>
+      </c>
+      <c r="AJ7">
+        <v>1500</v>
+      </c>
+      <c r="AK7">
+        <v>20.873999999999999</v>
+      </c>
+      <c r="AL7">
+        <v>20.925000000000001</v>
+      </c>
+      <c r="AM7">
+        <v>21.018000000000001</v>
+      </c>
+      <c r="AN7">
+        <v>21.010999999999999</v>
+      </c>
+      <c r="AO7">
+        <v>18.86</v>
+      </c>
+      <c r="AP7">
+        <v>24.832999999999998</v>
+      </c>
+      <c r="AQ7">
+        <v>24.591000000000001</v>
+      </c>
+      <c r="AR7">
+        <v>22.391999999999999</v>
+      </c>
+      <c r="AS7">
+        <v>21.065999999999999</v>
+      </c>
+      <c r="AT7">
+        <v>21.045999999999999</v>
+      </c>
+      <c r="AU7">
+        <v>20.85</v>
+      </c>
+      <c r="AV7">
+        <v>20.928999999999998</v>
+      </c>
+      <c r="AW7">
+        <v>21.023</v>
+      </c>
+      <c r="AX7">
+        <v>20.815000000000001</v>
+      </c>
+      <c r="AY7">
+        <v>20.962</v>
+      </c>
+      <c r="AZ7">
+        <v>20.86</v>
+      </c>
+      <c r="BA7">
+        <v>1</v>
+      </c>
+      <c r="BB7">
+        <v>1</v>
+      </c>
+      <c r="BC7">
+        <v>1</v>
+      </c>
+      <c r="BD7">
+        <v>0</v>
+      </c>
+      <c r="BE7">
+        <v>1</v>
+      </c>
+      <c r="BF7">
+        <v>0</v>
+      </c>
+      <c r="BG7">
+        <v>0</v>
+      </c>
+      <c r="BH7">
+        <v>0</v>
+      </c>
+      <c r="BI7">
+        <v>0</v>
+      </c>
+      <c r="BJ7">
+        <v>0</v>
+      </c>
+      <c r="BK7">
+        <v>0</v>
+      </c>
+      <c r="BL7">
+        <v>0</v>
+      </c>
+      <c r="BM7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>823</v>
+      </c>
+      <c r="B8" s="23">
+        <v>0.56099537037037039</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>1.9830000000000001</v>
+      </c>
+      <c r="I8">
+        <v>2.8730000000000002</v>
+      </c>
+      <c r="J8">
+        <v>5.556</v>
+      </c>
+      <c r="K8">
+        <v>2.758</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="0"/>
+        <v>13.169999999999998</v>
+      </c>
+      <c r="M8">
+        <v>500</v>
+      </c>
+      <c r="N8">
+        <v>200</v>
+      </c>
+      <c r="O8">
+        <v>200</v>
+      </c>
+      <c r="P8">
+        <v>100</v>
+      </c>
+      <c r="Q8">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="R8">
+        <v>0.40100000000000002</v>
+      </c>
+      <c r="S8">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="T8">
+        <v>-0.29299999999999998</v>
+      </c>
+      <c r="U8">
+        <v>1500</v>
+      </c>
+      <c r="V8">
+        <v>1500</v>
+      </c>
+      <c r="W8">
+        <v>1500</v>
+      </c>
+      <c r="X8">
+        <v>1500</v>
+      </c>
+      <c r="Y8">
+        <v>1500</v>
+      </c>
+      <c r="Z8">
+        <v>1500</v>
+      </c>
+      <c r="AA8">
+        <v>1500</v>
+      </c>
+      <c r="AB8">
+        <v>1500</v>
+      </c>
+      <c r="AC8">
+        <v>1500</v>
+      </c>
+      <c r="AD8">
+        <v>1500</v>
+      </c>
+      <c r="AE8">
+        <v>1500</v>
+      </c>
+      <c r="AF8">
+        <v>1500</v>
+      </c>
+      <c r="AG8">
+        <v>1500</v>
+      </c>
+      <c r="AH8">
+        <v>1500</v>
+      </c>
+      <c r="AI8">
+        <v>1500</v>
+      </c>
+      <c r="AJ8">
+        <v>1500</v>
+      </c>
+      <c r="AK8">
+        <v>33.274000000000001</v>
+      </c>
+      <c r="AL8">
+        <v>32.514000000000003</v>
+      </c>
+      <c r="AM8">
+        <v>43.92</v>
+      </c>
+      <c r="AN8">
+        <v>24.234000000000002</v>
+      </c>
+      <c r="AO8">
+        <v>19.815999999999999</v>
+      </c>
+      <c r="AP8">
+        <v>24.739000000000001</v>
+      </c>
+      <c r="AQ8">
+        <v>24.603999999999999</v>
+      </c>
+      <c r="AR8">
+        <v>30.073</v>
+      </c>
+      <c r="AS8">
+        <v>36.981000000000002</v>
+      </c>
+      <c r="AT8">
+        <v>42.470999999999997</v>
+      </c>
+      <c r="AU8">
+        <v>39.097000000000001</v>
+      </c>
+      <c r="AV8">
+        <v>33.854999999999997</v>
+      </c>
+      <c r="AW8">
+        <v>22.873999999999999</v>
+      </c>
+      <c r="AX8">
+        <v>22.6</v>
+      </c>
+      <c r="AY8">
+        <v>22.196999999999999</v>
+      </c>
+      <c r="AZ8">
+        <v>22.402000000000001</v>
+      </c>
+      <c r="BA8">
+        <v>1</v>
+      </c>
+      <c r="BB8">
+        <v>1</v>
+      </c>
+      <c r="BC8">
+        <v>1</v>
+      </c>
+      <c r="BD8">
+        <v>0</v>
+      </c>
+      <c r="BE8">
+        <v>1</v>
+      </c>
+      <c r="BF8">
+        <v>0</v>
+      </c>
+      <c r="BG8">
+        <v>0</v>
+      </c>
+      <c r="BH8">
+        <v>0</v>
+      </c>
+      <c r="BI8">
+        <v>0</v>
+      </c>
+      <c r="BJ8">
+        <v>0</v>
+      </c>
+      <c r="BK8">
+        <v>0</v>
+      </c>
+      <c r="BL8">
+        <v>0</v>
+      </c>
+      <c r="BM8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>824</v>
+      </c>
+      <c r="B9" s="23">
+        <v>0.52262731481481484</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>1.9810000000000001</v>
+      </c>
+      <c r="I9">
+        <v>2.8730000000000002</v>
+      </c>
+      <c r="J9">
+        <v>2.7810000000000001</v>
+      </c>
+      <c r="K9">
+        <v>1.381</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="0"/>
+        <v>9.016</v>
+      </c>
+      <c r="M9">
+        <v>500</v>
+      </c>
+      <c r="N9">
+        <v>200</v>
+      </c>
+      <c r="O9">
+        <v>200</v>
+      </c>
+      <c r="P9">
+        <v>100</v>
+      </c>
+      <c r="Q9">
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="R9">
+        <v>0.38300000000000001</v>
+      </c>
+      <c r="S9">
+        <v>-0.23300000000000001</v>
+      </c>
+      <c r="T9">
+        <v>-0.317</v>
+      </c>
+      <c r="U9">
+        <v>1500</v>
+      </c>
+      <c r="V9">
+        <v>1500</v>
+      </c>
+      <c r="W9">
+        <v>1500</v>
+      </c>
+      <c r="X9">
+        <v>1500</v>
+      </c>
+      <c r="Y9">
+        <v>1500</v>
+      </c>
+      <c r="Z9">
+        <v>1500</v>
+      </c>
+      <c r="AA9">
+        <v>1500</v>
+      </c>
+      <c r="AB9">
+        <v>1500</v>
+      </c>
+      <c r="AC9">
+        <v>1500</v>
+      </c>
+      <c r="AD9">
+        <v>1500</v>
+      </c>
+      <c r="AE9">
+        <v>1500</v>
+      </c>
+      <c r="AF9">
+        <v>1500</v>
+      </c>
+      <c r="AG9">
+        <v>1500</v>
+      </c>
+      <c r="AH9">
+        <v>1500</v>
+      </c>
+      <c r="AI9">
+        <v>1500</v>
+      </c>
+      <c r="AJ9">
+        <v>1500</v>
+      </c>
+      <c r="AK9">
+        <v>20.971</v>
+      </c>
+      <c r="AL9">
+        <v>20.718</v>
+      </c>
+      <c r="AM9">
+        <v>20.951000000000001</v>
+      </c>
+      <c r="AN9">
+        <v>20.83</v>
+      </c>
+      <c r="AO9">
+        <v>18.888999999999999</v>
+      </c>
+      <c r="AP9">
+        <v>24.991</v>
+      </c>
+      <c r="AQ9">
+        <v>24.759</v>
+      </c>
+      <c r="AR9">
+        <v>22.398</v>
+      </c>
+      <c r="AS9">
+        <v>21.032</v>
+      </c>
+      <c r="AT9">
+        <v>20.963000000000001</v>
+      </c>
+      <c r="AU9">
+        <v>20.91</v>
+      </c>
+      <c r="AV9">
+        <v>21.073</v>
+      </c>
+      <c r="AW9">
+        <v>20.884</v>
+      </c>
+      <c r="AX9">
+        <v>20.704000000000001</v>
+      </c>
+      <c r="AY9">
+        <v>20.826000000000001</v>
+      </c>
+      <c r="AZ9">
+        <v>20.736000000000001</v>
+      </c>
+      <c r="BA9">
+        <v>1</v>
+      </c>
+      <c r="BB9">
+        <v>1</v>
+      </c>
+      <c r="BC9">
+        <v>1</v>
+      </c>
+      <c r="BD9">
+        <v>0</v>
+      </c>
+      <c r="BE9">
+        <v>1</v>
+      </c>
+      <c r="BF9">
+        <v>0</v>
+      </c>
+      <c r="BG9">
+        <v>0</v>
+      </c>
+      <c r="BH9">
+        <v>0</v>
+      </c>
+      <c r="BI9">
+        <v>0</v>
+      </c>
+      <c r="BJ9">
+        <v>0</v>
+      </c>
+      <c r="BK9">
+        <v>0</v>
+      </c>
+      <c r="BL9">
+        <v>0</v>
+      </c>
+      <c r="BM9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>825</v>
+      </c>
+      <c r="B10" s="23">
+        <v>0.68175925925925929</v>
+      </c>
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1.982</v>
+      </c>
+      <c r="I10">
+        <v>2.8690000000000002</v>
+      </c>
+      <c r="J10">
+        <v>1.399</v>
+      </c>
+      <c r="K10">
+        <v>0.69</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="0"/>
+        <v>6.9399999999999995</v>
+      </c>
+      <c r="M10">
+        <v>500</v>
+      </c>
+      <c r="N10">
+        <v>200</v>
+      </c>
+      <c r="O10">
+        <v>200</v>
+      </c>
+      <c r="P10">
+        <v>100</v>
+      </c>
+      <c r="Q10">
+        <v>0.70099999999999996</v>
+      </c>
+      <c r="R10">
+        <v>0.39900000000000002</v>
+      </c>
+      <c r="S10">
+        <v>-0.29899999999999999</v>
+      </c>
+      <c r="T10">
+        <v>-0.30099999999999999</v>
+      </c>
+      <c r="U10">
+        <v>1500</v>
+      </c>
+      <c r="V10">
+        <v>1500</v>
+      </c>
+      <c r="W10">
+        <v>1500</v>
+      </c>
+      <c r="X10">
+        <v>1500</v>
+      </c>
+      <c r="Y10">
+        <v>1500</v>
+      </c>
+      <c r="Z10">
+        <v>1500</v>
+      </c>
+      <c r="AA10">
+        <v>1500</v>
+      </c>
+      <c r="AB10">
+        <v>1500</v>
+      </c>
+      <c r="AC10">
+        <v>1500</v>
+      </c>
+      <c r="AD10">
+        <v>1500</v>
+      </c>
+      <c r="AE10">
+        <v>1500</v>
+      </c>
+      <c r="AF10">
+        <v>1500</v>
+      </c>
+      <c r="AG10">
+        <v>1500</v>
+      </c>
+      <c r="AH10">
+        <v>1500</v>
+      </c>
+      <c r="AI10">
+        <v>1500</v>
+      </c>
+      <c r="AJ10">
+        <v>1500</v>
+      </c>
+      <c r="AK10">
+        <v>20.853000000000002</v>
+      </c>
+      <c r="AL10">
+        <v>20.786000000000001</v>
+      </c>
+      <c r="AM10">
+        <v>20.949000000000002</v>
+      </c>
+      <c r="AN10">
+        <v>20.873999999999999</v>
+      </c>
+      <c r="AO10">
+        <v>18.873000000000001</v>
+      </c>
+      <c r="AP10">
+        <v>25.024000000000001</v>
+      </c>
+      <c r="AQ10">
+        <v>24.71</v>
+      </c>
+      <c r="AR10">
+        <v>22.398</v>
+      </c>
+      <c r="AS10">
+        <v>21.036000000000001</v>
+      </c>
+      <c r="AT10">
+        <v>20.966999999999999</v>
+      </c>
+      <c r="AU10">
+        <v>20.88</v>
+      </c>
+      <c r="AV10">
+        <v>21.052</v>
+      </c>
+      <c r="AW10">
+        <v>20.933</v>
+      </c>
+      <c r="AX10">
+        <v>20.748999999999999</v>
+      </c>
+      <c r="AY10">
+        <v>20.890999999999998</v>
+      </c>
+      <c r="AZ10">
+        <v>20.785</v>
+      </c>
+      <c r="BA10">
+        <v>1</v>
+      </c>
+      <c r="BB10">
+        <v>1</v>
+      </c>
+      <c r="BC10">
+        <v>1</v>
+      </c>
+      <c r="BD10">
+        <v>0</v>
+      </c>
+      <c r="BE10">
+        <v>1</v>
+      </c>
+      <c r="BF10">
+        <v>0</v>
+      </c>
+      <c r="BG10">
+        <v>0</v>
+      </c>
+      <c r="BH10">
+        <v>0</v>
+      </c>
+      <c r="BI10">
+        <v>0</v>
+      </c>
+      <c r="BJ10">
+        <v>0</v>
+      </c>
+      <c r="BK10">
+        <v>0</v>
+      </c>
+      <c r="BL10">
+        <v>0</v>
+      </c>
+      <c r="BM10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>826</v>
+      </c>
+      <c r="B11" s="23">
+        <v>0.5037962962962963</v>
+      </c>
+      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0.995</v>
+      </c>
+      <c r="I11">
+        <v>1.4339999999999999</v>
+      </c>
+      <c r="J11">
+        <v>1.395</v>
+      </c>
+      <c r="K11">
+        <v>0.69099999999999995</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>4.5149999999999997</v>
+      </c>
+      <c r="M11">
+        <v>500</v>
+      </c>
+      <c r="N11">
+        <v>200</v>
+      </c>
+      <c r="O11">
+        <v>200</v>
+      </c>
+      <c r="P11">
+        <v>100</v>
+      </c>
+      <c r="Q11">
+        <v>0.69499999999999995</v>
+      </c>
+      <c r="R11">
+        <v>0.39600000000000002</v>
+      </c>
+      <c r="S11">
+        <v>-0.38700000000000001</v>
+      </c>
+      <c r="T11">
+        <v>-0.29899999999999999</v>
+      </c>
+      <c r="U11">
+        <v>1500</v>
+      </c>
+      <c r="V11">
+        <v>1500</v>
+      </c>
+      <c r="W11">
+        <v>1500</v>
+      </c>
+      <c r="X11">
+        <v>1500</v>
+      </c>
+      <c r="Y11">
+        <v>1500</v>
+      </c>
+      <c r="Z11">
+        <v>1500</v>
+      </c>
+      <c r="AA11">
+        <v>1500</v>
+      </c>
+      <c r="AB11">
+        <v>1500</v>
+      </c>
+      <c r="AC11">
+        <v>1500</v>
+      </c>
+      <c r="AD11">
+        <v>1500</v>
+      </c>
+      <c r="AE11">
+        <v>1500</v>
+      </c>
+      <c r="AF11">
+        <v>1500</v>
+      </c>
+      <c r="AG11">
+        <v>1500</v>
+      </c>
+      <c r="AH11">
+        <v>1500</v>
+      </c>
+      <c r="AI11">
+        <v>1500</v>
+      </c>
+      <c r="AJ11">
+        <v>1500</v>
+      </c>
+      <c r="AK11">
+        <v>20.855</v>
+      </c>
+      <c r="AL11">
+        <v>20.702000000000002</v>
+      </c>
+      <c r="AM11">
+        <v>20.902999999999999</v>
+      </c>
+      <c r="AN11">
+        <v>20.754000000000001</v>
+      </c>
+      <c r="AO11">
+        <v>18.815000000000001</v>
+      </c>
+      <c r="AP11">
+        <v>23.187999999999999</v>
+      </c>
+      <c r="AQ11">
+        <v>22.864000000000001</v>
+      </c>
+      <c r="AR11">
+        <v>22.387</v>
+      </c>
+      <c r="AS11">
+        <v>20.905999999999999</v>
+      </c>
+      <c r="AT11">
+        <v>20.934999999999999</v>
+      </c>
+      <c r="AU11">
+        <v>20.835999999999999</v>
+      </c>
+      <c r="AV11">
+        <v>21.026</v>
+      </c>
+      <c r="AW11">
+        <v>20.809000000000001</v>
+      </c>
+      <c r="AX11">
+        <v>20.652999999999999</v>
+      </c>
+      <c r="AY11">
+        <v>20.815999999999999</v>
+      </c>
+      <c r="AZ11">
+        <v>20.710999999999999</v>
+      </c>
+      <c r="BA11">
+        <v>1</v>
+      </c>
+      <c r="BB11">
+        <v>1</v>
+      </c>
+      <c r="BC11">
+        <v>1</v>
+      </c>
+      <c r="BD11">
+        <v>0</v>
+      </c>
+      <c r="BE11">
+        <v>1</v>
+      </c>
+      <c r="BF11">
+        <v>0</v>
+      </c>
+      <c r="BG11">
+        <v>0</v>
+      </c>
+      <c r="BH11">
+        <v>0</v>
+      </c>
+      <c r="BI11">
+        <v>0</v>
+      </c>
+      <c r="BJ11">
+        <v>0</v>
+      </c>
+      <c r="BK11">
+        <v>0</v>
+      </c>
+      <c r="BL11">
+        <v>0</v>
+      </c>
+      <c r="BM11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>827</v>
+      </c>
+      <c r="B12" s="23">
+        <v>0.67587962962962966</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>3.9590000000000001</v>
+      </c>
+      <c r="I12">
+        <v>5.718</v>
+      </c>
+      <c r="J12">
+        <v>2.786</v>
+      </c>
+      <c r="K12">
+        <v>1.3819999999999999</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="0"/>
+        <v>13.844999999999999</v>
+      </c>
+      <c r="M12">
+        <v>500</v>
+      </c>
+      <c r="N12">
+        <v>200</v>
+      </c>
+      <c r="O12">
+        <v>200</v>
+      </c>
+      <c r="P12">
+        <v>100</v>
+      </c>
+      <c r="Q12">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="R12">
+        <v>0.39100000000000001</v>
+      </c>
+      <c r="S12">
+        <v>6.2E-2</v>
+      </c>
+      <c r="T12">
+        <v>-0.29299999999999998</v>
+      </c>
+      <c r="U12">
+        <v>1500</v>
+      </c>
+      <c r="V12">
+        <v>1500</v>
+      </c>
+      <c r="W12">
+        <v>1500</v>
+      </c>
+      <c r="X12">
+        <v>1500</v>
+      </c>
+      <c r="Y12">
+        <v>1500</v>
+      </c>
+      <c r="Z12">
+        <v>1500</v>
+      </c>
+      <c r="AA12">
+        <v>1500</v>
+      </c>
+      <c r="AB12">
+        <v>1500</v>
+      </c>
+      <c r="AC12">
+        <v>1500</v>
+      </c>
+      <c r="AD12">
+        <v>1500</v>
+      </c>
+      <c r="AE12">
+        <v>1500</v>
+      </c>
+      <c r="AF12">
+        <v>1500</v>
+      </c>
+      <c r="AG12">
+        <v>1500</v>
+      </c>
+      <c r="AH12">
+        <v>1500</v>
+      </c>
+      <c r="AI12">
+        <v>1500</v>
+      </c>
+      <c r="AJ12">
+        <v>1500</v>
+      </c>
+      <c r="AK12">
+        <v>38.015000000000001</v>
+      </c>
+      <c r="AL12">
+        <v>34.933999999999997</v>
+      </c>
+      <c r="AM12">
+        <v>49.42</v>
+      </c>
+      <c r="AN12">
+        <v>23.440999999999999</v>
+      </c>
+      <c r="AO12">
+        <v>19.760000000000002</v>
+      </c>
+      <c r="AP12">
+        <v>24.747</v>
+      </c>
+      <c r="AQ12">
+        <v>24.574000000000002</v>
+      </c>
+      <c r="AR12">
+        <v>37.11</v>
+      </c>
+      <c r="AS12">
+        <v>45.844000000000001</v>
+      </c>
+      <c r="AT12">
+        <v>48.715000000000003</v>
+      </c>
+      <c r="AU12">
+        <v>46.834000000000003</v>
+      </c>
+      <c r="AV12">
+        <v>44.712000000000003</v>
+      </c>
+      <c r="AW12">
+        <v>22.701000000000001</v>
+      </c>
+      <c r="AX12">
+        <v>22.417999999999999</v>
+      </c>
+      <c r="AY12">
+        <v>22.122</v>
+      </c>
+      <c r="AZ12">
+        <v>22.291</v>
+      </c>
+      <c r="BA12">
+        <v>1</v>
+      </c>
+      <c r="BB12">
+        <v>1</v>
+      </c>
+      <c r="BC12">
+        <v>1</v>
+      </c>
+      <c r="BD12">
+        <v>0</v>
+      </c>
+      <c r="BE12">
+        <v>1</v>
+      </c>
+      <c r="BF12">
+        <v>0</v>
+      </c>
+      <c r="BG12">
+        <v>0</v>
+      </c>
+      <c r="BH12">
+        <v>0</v>
+      </c>
+      <c r="BI12">
+        <v>0</v>
+      </c>
+      <c r="BJ12">
+        <v>0</v>
+      </c>
+      <c r="BK12">
+        <v>0</v>
+      </c>
+      <c r="BL12">
+        <v>0</v>
+      </c>
+      <c r="BM12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>686</v>
+      </c>
+      <c r="B13" s="23">
+        <v>0.55775462962962963</v>
+      </c>
+      <c r="C13">
+        <v>19</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>2.9670000000000001</v>
+      </c>
+      <c r="I13">
+        <v>2.871</v>
+      </c>
+      <c r="J13">
+        <v>2.7890000000000001</v>
+      </c>
+      <c r="K13">
+        <v>1.38</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="0"/>
+        <v>10.007000000000001</v>
+      </c>
+      <c r="M13">
+        <v>500</v>
+      </c>
+      <c r="N13">
+        <v>200</v>
+      </c>
+      <c r="O13">
+        <v>200</v>
+      </c>
+      <c r="P13">
+        <v>100</v>
+      </c>
+      <c r="Q13">
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="R13">
+        <v>0.39600000000000002</v>
+      </c>
+      <c r="S13">
+        <v>-0.13900000000000001</v>
+      </c>
+      <c r="T13">
+        <v>-0.314</v>
+      </c>
+      <c r="U13">
+        <v>1500</v>
+      </c>
+      <c r="V13">
+        <v>1500</v>
+      </c>
+      <c r="W13">
+        <v>1500</v>
+      </c>
+      <c r="X13">
+        <v>1500</v>
+      </c>
+      <c r="Y13">
+        <v>1500</v>
+      </c>
+      <c r="Z13">
+        <v>1500</v>
+      </c>
+      <c r="AA13">
+        <v>1500</v>
+      </c>
+      <c r="AB13">
+        <v>1500</v>
+      </c>
+      <c r="AC13">
+        <v>1500</v>
+      </c>
+      <c r="AD13">
+        <v>1500</v>
+      </c>
+      <c r="AE13">
+        <v>1500</v>
+      </c>
+      <c r="AF13">
+        <v>1500</v>
+      </c>
+      <c r="AG13">
+        <v>1500</v>
+      </c>
+      <c r="AH13">
+        <v>1500</v>
+      </c>
+      <c r="AI13">
+        <v>1500</v>
+      </c>
+      <c r="AJ13">
+        <v>1500</v>
+      </c>
+      <c r="AK13">
+        <v>27.007999999999999</v>
+      </c>
+      <c r="AL13">
+        <v>21.03</v>
+      </c>
+      <c r="AM13">
+        <v>21.693000000000001</v>
+      </c>
+      <c r="AN13">
+        <v>21.242999999999999</v>
+      </c>
+      <c r="AO13">
+        <v>19.3</v>
+      </c>
+      <c r="AP13">
+        <v>24.405999999999999</v>
+      </c>
+      <c r="AQ13">
+        <v>24.085999999999999</v>
+      </c>
+      <c r="AR13">
+        <v>29.126000000000001</v>
+      </c>
+      <c r="AS13">
+        <v>21.548999999999999</v>
+      </c>
+      <c r="AT13">
+        <v>21.38</v>
+      </c>
+      <c r="AU13">
+        <v>22.134</v>
+      </c>
+      <c r="AV13">
+        <v>23.260999999999999</v>
+      </c>
+      <c r="AW13">
+        <v>21.247</v>
+      </c>
+      <c r="AX13">
+        <v>21.058</v>
+      </c>
+      <c r="AY13">
+        <v>21.236999999999998</v>
+      </c>
+      <c r="AZ13">
+        <v>21.102</v>
+      </c>
+      <c r="BA13">
+        <v>1</v>
+      </c>
+      <c r="BB13">
+        <v>1</v>
+      </c>
+      <c r="BC13">
+        <v>1</v>
+      </c>
+      <c r="BD13">
+        <v>0</v>
+      </c>
+      <c r="BE13">
+        <v>1</v>
+      </c>
+      <c r="BF13">
+        <v>0</v>
+      </c>
+      <c r="BG13">
+        <v>0</v>
+      </c>
+      <c r="BH13">
+        <v>0</v>
+      </c>
+      <c r="BI13">
+        <v>0</v>
+      </c>
+      <c r="BJ13">
+        <v>0</v>
+      </c>
+      <c r="BK13">
+        <v>0</v>
+      </c>
+      <c r="BL13">
+        <v>0</v>
+      </c>
+      <c r="BM13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>828</v>
+      </c>
+      <c r="B14" s="23">
+        <v>0.72422453703703704</v>
+      </c>
+      <c r="C14">
+        <v>9</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
+        <v>0.99</v>
+      </c>
+      <c r="I14">
+        <v>2.86</v>
+      </c>
+      <c r="J14">
+        <v>2.778</v>
+      </c>
+      <c r="K14">
+        <v>1.383</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="0"/>
+        <v>8.0109999999999992</v>
+      </c>
+      <c r="M14">
+        <v>500</v>
+      </c>
+      <c r="N14">
+        <v>200</v>
+      </c>
+      <c r="O14">
+        <v>200</v>
+      </c>
+      <c r="P14">
+        <v>100</v>
+      </c>
+      <c r="Q14">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="R14">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="S14">
+        <v>-0.22600000000000001</v>
+      </c>
+      <c r="T14">
+        <v>-0.28199999999999997</v>
+      </c>
+      <c r="U14">
+        <v>1500</v>
+      </c>
+      <c r="V14">
+        <v>1500</v>
+      </c>
+      <c r="W14">
+        <v>1500</v>
+      </c>
+      <c r="X14">
+        <v>1500</v>
+      </c>
+      <c r="Y14">
+        <v>1500</v>
+      </c>
+      <c r="Z14">
+        <v>1500</v>
+      </c>
+      <c r="AA14">
+        <v>1500</v>
+      </c>
+      <c r="AB14">
+        <v>1500</v>
+      </c>
+      <c r="AC14">
+        <v>1500</v>
+      </c>
+      <c r="AD14">
+        <v>1500</v>
+      </c>
+      <c r="AE14">
+        <v>1500</v>
+      </c>
+      <c r="AF14">
+        <v>1500</v>
+      </c>
+      <c r="AG14">
+        <v>1500</v>
+      </c>
+      <c r="AH14">
+        <v>1500</v>
+      </c>
+      <c r="AI14">
+        <v>1500</v>
+      </c>
+      <c r="AJ14">
+        <v>1500</v>
+      </c>
+      <c r="AK14">
+        <v>27.495000000000001</v>
+      </c>
+      <c r="AL14">
+        <v>27.335000000000001</v>
+      </c>
+      <c r="AM14">
+        <v>30.024000000000001</v>
+      </c>
+      <c r="AN14">
+        <v>22.646999999999998</v>
+      </c>
+      <c r="AO14">
+        <v>20.405999999999999</v>
+      </c>
+      <c r="AP14">
+        <v>24.966000000000001</v>
+      </c>
+      <c r="AQ14">
+        <v>24.79</v>
+      </c>
+      <c r="AR14">
+        <v>26.724</v>
+      </c>
+      <c r="AS14">
+        <v>28.539000000000001</v>
+      </c>
+      <c r="AT14">
+        <v>29.795999999999999</v>
+      </c>
+      <c r="AU14">
+        <v>29.161000000000001</v>
+      </c>
+      <c r="AV14">
+        <v>27.957000000000001</v>
+      </c>
+      <c r="AW14">
+        <v>23.061</v>
+      </c>
+      <c r="AX14">
+        <v>22.806000000000001</v>
+      </c>
+      <c r="AY14">
+        <v>22.652000000000001</v>
+      </c>
+      <c r="AZ14">
+        <v>22.73</v>
+      </c>
+      <c r="BA14">
+        <v>1</v>
+      </c>
+      <c r="BB14">
+        <v>1</v>
+      </c>
+      <c r="BC14">
+        <v>1</v>
+      </c>
+      <c r="BD14">
+        <v>0</v>
+      </c>
+      <c r="BE14">
+        <v>1</v>
+      </c>
+      <c r="BF14">
+        <v>0</v>
+      </c>
+      <c r="BG14">
+        <v>0</v>
+      </c>
+      <c r="BH14">
+        <v>0</v>
+      </c>
+      <c r="BI14">
+        <v>0</v>
+      </c>
+      <c r="BJ14">
+        <v>0</v>
+      </c>
+      <c r="BK14">
+        <v>0</v>
+      </c>
+      <c r="BL14">
+        <v>0</v>
+      </c>
+      <c r="BM14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>829</v>
+      </c>
+      <c r="B15" s="23">
+        <v>0.41075231481481483</v>
+      </c>
+      <c r="C15">
+        <v>7</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15">
+        <v>0.99</v>
+      </c>
+      <c r="I15">
+        <v>1.4419999999999999</v>
+      </c>
+      <c r="J15">
+        <v>2.786</v>
+      </c>
+      <c r="K15">
+        <v>1.381</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="0"/>
+        <v>6.5990000000000002</v>
+      </c>
+      <c r="M15">
+        <v>500</v>
+      </c>
+      <c r="N15">
+        <v>200</v>
+      </c>
+      <c r="O15">
+        <v>200</v>
+      </c>
+      <c r="P15">
+        <v>100</v>
+      </c>
+      <c r="Q15">
+        <v>0.69499999999999995</v>
+      </c>
+      <c r="R15">
+        <v>0.39700000000000002</v>
+      </c>
+      <c r="S15">
+        <v>-0.29899999999999999</v>
+      </c>
+      <c r="T15">
+        <v>-0.30299999999999999</v>
+      </c>
+      <c r="U15">
+        <v>1500</v>
+      </c>
+      <c r="V15">
+        <v>1500</v>
+      </c>
+      <c r="W15">
+        <v>1500</v>
+      </c>
+      <c r="X15">
+        <v>1500</v>
+      </c>
+      <c r="Y15">
+        <v>1500</v>
+      </c>
+      <c r="Z15">
+        <v>1500</v>
+      </c>
+      <c r="AA15">
+        <v>1500</v>
+      </c>
+      <c r="AB15">
+        <v>1500</v>
+      </c>
+      <c r="AC15">
+        <v>1500</v>
+      </c>
+      <c r="AD15">
+        <v>1500</v>
+      </c>
+      <c r="AE15">
+        <v>1500</v>
+      </c>
+      <c r="AF15">
+        <v>1500</v>
+      </c>
+      <c r="AG15">
+        <v>1500</v>
+      </c>
+      <c r="AH15">
+        <v>1500</v>
+      </c>
+      <c r="AI15">
+        <v>1500</v>
+      </c>
+      <c r="AJ15">
+        <v>1500</v>
+      </c>
+      <c r="AK15">
+        <v>21.375</v>
+      </c>
+      <c r="AL15">
+        <v>21.209</v>
+      </c>
+      <c r="AM15">
+        <v>21.423999999999999</v>
+      </c>
+      <c r="AN15">
+        <v>21.198</v>
+      </c>
+      <c r="AO15">
+        <v>19.128</v>
+      </c>
+      <c r="AP15">
+        <v>24.588999999999999</v>
+      </c>
+      <c r="AQ15">
+        <v>24.321000000000002</v>
+      </c>
+      <c r="AR15">
+        <v>22.806999999999999</v>
+      </c>
+      <c r="AS15">
+        <v>21.539000000000001</v>
+      </c>
+      <c r="AT15">
+        <v>21.484000000000002</v>
+      </c>
+      <c r="AU15">
+        <v>21.379000000000001</v>
+      </c>
+      <c r="AV15">
+        <v>21.475000000000001</v>
+      </c>
+      <c r="AW15">
+        <v>21.298999999999999</v>
+      </c>
+      <c r="AX15">
+        <v>21.097000000000001</v>
+      </c>
+      <c r="AY15">
+        <v>21.177</v>
+      </c>
+      <c r="AZ15">
+        <v>21.087</v>
+      </c>
+      <c r="BA15">
+        <v>1</v>
+      </c>
+      <c r="BB15">
+        <v>1</v>
+      </c>
+      <c r="BC15">
+        <v>1</v>
+      </c>
+      <c r="BD15">
+        <v>0</v>
+      </c>
+      <c r="BE15">
+        <v>1</v>
+      </c>
+      <c r="BF15">
+        <v>0</v>
+      </c>
+      <c r="BG15">
+        <v>0</v>
+      </c>
+      <c r="BH15">
+        <v>0</v>
+      </c>
+      <c r="BI15">
+        <v>0</v>
+      </c>
+      <c r="BJ15">
+        <v>0</v>
+      </c>
+      <c r="BK15">
+        <v>0</v>
+      </c>
+      <c r="BL15">
+        <v>0</v>
+      </c>
+      <c r="BM15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>830</v>
+      </c>
+      <c r="B16" s="23">
+        <v>0.57916666666666672</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>0.99</v>
+      </c>
+      <c r="I16">
+        <v>1.4379999999999999</v>
+      </c>
+      <c r="J16">
+        <v>1.3919999999999999</v>
+      </c>
+      <c r="K16">
+        <v>0.69099999999999995</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="0"/>
+        <v>4.5110000000000001</v>
+      </c>
+      <c r="M16">
+        <v>500</v>
+      </c>
+      <c r="N16">
+        <v>200</v>
+      </c>
+      <c r="O16">
+        <v>200</v>
+      </c>
+      <c r="P16">
+        <v>100</v>
+      </c>
+      <c r="Q16">
+        <v>0.70399999999999996</v>
+      </c>
+      <c r="R16">
+        <v>0.39600000000000002</v>
+      </c>
+      <c r="S16">
+        <v>-0.36799999999999999</v>
+      </c>
+      <c r="T16">
+        <v>-0.29799999999999999</v>
+      </c>
+      <c r="U16">
+        <v>1500</v>
+      </c>
+      <c r="V16">
+        <v>1500</v>
+      </c>
+      <c r="W16">
+        <v>1500</v>
+      </c>
+      <c r="X16">
+        <v>1500</v>
+      </c>
+      <c r="Y16">
+        <v>1500</v>
+      </c>
+      <c r="Z16">
+        <v>1500</v>
+      </c>
+      <c r="AA16">
+        <v>1500</v>
+      </c>
+      <c r="AB16">
+        <v>1500</v>
+      </c>
+      <c r="AC16">
+        <v>1500</v>
+      </c>
+      <c r="AD16">
+        <v>1500</v>
+      </c>
+      <c r="AE16">
+        <v>1500</v>
+      </c>
+      <c r="AF16">
+        <v>1500</v>
+      </c>
+      <c r="AG16">
+        <v>1500</v>
+      </c>
+      <c r="AH16">
+        <v>1500</v>
+      </c>
+      <c r="AI16">
+        <v>1500</v>
+      </c>
+      <c r="AJ16">
+        <v>1500</v>
+      </c>
+      <c r="AK16">
+        <v>27.341000000000001</v>
+      </c>
+      <c r="AL16">
+        <v>26.523</v>
+      </c>
+      <c r="AM16">
+        <v>30.777000000000001</v>
+      </c>
+      <c r="AN16">
+        <v>21.861999999999998</v>
+      </c>
+      <c r="AO16">
+        <v>20.027999999999999</v>
+      </c>
+      <c r="AP16">
+        <v>25.474</v>
+      </c>
+      <c r="AQ16">
+        <v>25.346</v>
+      </c>
+      <c r="AR16">
+        <v>27.632999999999999</v>
+      </c>
+      <c r="AS16">
+        <v>29.855</v>
+      </c>
+      <c r="AT16">
+        <v>30.751000000000001</v>
+      </c>
+      <c r="AU16">
+        <v>30.462</v>
+      </c>
+      <c r="AV16">
+        <v>29.603000000000002</v>
+      </c>
+      <c r="AW16">
+        <v>22.361999999999998</v>
+      </c>
+      <c r="AX16">
+        <v>22.137</v>
+      </c>
+      <c r="AY16">
+        <v>22.135999999999999</v>
+      </c>
+      <c r="AZ16">
+        <v>22.14</v>
+      </c>
+      <c r="BA16">
+        <v>1</v>
+      </c>
+      <c r="BB16">
+        <v>1</v>
+      </c>
+      <c r="BC16">
+        <v>1</v>
+      </c>
+      <c r="BD16">
+        <v>0</v>
+      </c>
+      <c r="BE16">
+        <v>1</v>
+      </c>
+      <c r="BF16">
+        <v>0</v>
+      </c>
+      <c r="BG16">
+        <v>0</v>
+      </c>
+      <c r="BH16">
+        <v>0</v>
+      </c>
+      <c r="BI16">
+        <v>0</v>
+      </c>
+      <c r="BJ16">
+        <v>0</v>
+      </c>
+      <c r="BK16">
+        <v>0</v>
+      </c>
+      <c r="BL16">
+        <v>0</v>
+      </c>
+      <c r="BM16">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>